<commit_message>
refactor: delete duplicated geometry
</commit_message>
<xml_diff>
--- a/project/config/profile_config_file.xlsx
+++ b/project/config/profile_config_file.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsochacki\Desktop\Python\Tkinter\production-counting\project\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{534B9F16-FECA-456B-AC0E-103CE09484FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE0C3EA-950A-4F36-82E9-3AB764CEEB0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-195" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="profile_config" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="176">
   <si>
     <t>GP8280</t>
   </si>
@@ -837,7 +837,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C567"/>
+  <dimension ref="A1:C566"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" customWidth="1"/>
@@ -5578,29 +5578,29 @@
     </row>
     <row r="431" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A431">
-        <v>416182</v>
+        <v>416070</v>
       </c>
       <c r="B431" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C431">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="432" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A432">
-        <v>416070</v>
+        <v>416069</v>
       </c>
       <c r="B432" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C432">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="433" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A433">
-        <v>416069</v>
+      <c r="A433" t="s">
+        <v>124</v>
       </c>
       <c r="B433" s="1" t="s">
         <v>1</v>
@@ -5610,8 +5610,8 @@
       </c>
     </row>
     <row r="434" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A434" t="s">
-        <v>124</v>
+      <c r="A434">
+        <v>406340</v>
       </c>
       <c r="B434" s="1" t="s">
         <v>1</v>
@@ -5622,7 +5622,7 @@
     </row>
     <row r="435" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A435">
-        <v>406340</v>
+        <v>416301</v>
       </c>
       <c r="B435" s="1" t="s">
         <v>1</v>
@@ -5633,35 +5633,35 @@
     </row>
     <row r="436" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A436">
-        <v>416301</v>
+        <v>416119</v>
       </c>
       <c r="B436" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C436">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="437" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A437">
-        <v>416119</v>
+        <v>406081</v>
       </c>
       <c r="B437" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C437">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="438" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A438">
-        <v>406081</v>
+        <v>416068</v>
       </c>
       <c r="B438" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C438">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="439" spans="1:3" x14ac:dyDescent="0.25">
@@ -5669,26 +5669,26 @@
         <v>416068</v>
       </c>
       <c r="B439" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C439">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="440" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A440">
-        <v>416068</v>
+        <v>736315</v>
       </c>
       <c r="B440" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C440">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="441" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A441">
-        <v>736315</v>
+        <v>736334</v>
       </c>
       <c r="B441" s="1" t="s">
         <v>1</v>
@@ -5698,8 +5698,8 @@
       </c>
     </row>
     <row r="442" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A442">
-        <v>736334</v>
+      <c r="A442" t="s">
+        <v>125</v>
       </c>
       <c r="B442" s="1" t="s">
         <v>1</v>
@@ -5709,8 +5709,8 @@
       </c>
     </row>
     <row r="443" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A443" t="s">
-        <v>125</v>
+      <c r="A443">
+        <v>406307</v>
       </c>
       <c r="B443" s="1" t="s">
         <v>1</v>
@@ -5721,7 +5721,7 @@
     </row>
     <row r="444" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A444">
-        <v>406307</v>
+        <v>466400</v>
       </c>
       <c r="B444" s="1" t="s">
         <v>1</v>
@@ -5732,13 +5732,13 @@
     </row>
     <row r="445" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A445">
-        <v>466400</v>
+        <v>416139</v>
       </c>
       <c r="B445" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C445">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="446" spans="1:3" x14ac:dyDescent="0.25">
@@ -5746,7 +5746,7 @@
         <v>416139</v>
       </c>
       <c r="B446" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C446">
         <v>80</v>
@@ -5754,7 +5754,7 @@
     </row>
     <row r="447" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A447">
-        <v>416139</v>
+        <v>416148</v>
       </c>
       <c r="B447" s="1" t="s">
         <v>1</v>
@@ -5764,30 +5764,30 @@
       </c>
     </row>
     <row r="448" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A448">
-        <v>416148</v>
+      <c r="A448" t="s">
+        <v>126</v>
       </c>
       <c r="B448" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C448">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="449" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B449" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C449">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="450" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B450" s="1" t="s">
         <v>1</v>
@@ -5798,7 +5798,7 @@
     </row>
     <row r="451" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B451" s="1" t="s">
         <v>1</v>
@@ -5809,40 +5809,40 @@
     </row>
     <row r="452" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B452" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C452">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="453" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B453" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C453">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="454" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B454" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C454">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="455" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B455" s="1" t="s">
         <v>1</v>
@@ -5852,30 +5852,30 @@
       </c>
     </row>
     <row r="456" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A456" t="s">
-        <v>133</v>
+      <c r="A456">
+        <v>406310</v>
       </c>
       <c r="B456" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C456">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="457" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A457" t="s">
+        <v>134</v>
+      </c>
+      <c r="B457" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C457">
         <v>80</v>
       </c>
     </row>
-    <row r="457" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A457">
-        <v>406310</v>
-      </c>
-      <c r="B457" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C457">
-        <v>90</v>
-      </c>
-    </row>
     <row r="458" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A458" t="s">
-        <v>134</v>
+      <c r="A458">
+        <v>416180</v>
       </c>
       <c r="B458" s="1" t="s">
         <v>1</v>
@@ -5886,7 +5886,7 @@
     </row>
     <row r="459" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A459">
-        <v>416180</v>
+        <v>606180</v>
       </c>
       <c r="B459" s="1" t="s">
         <v>1</v>
@@ -5897,7 +5897,7 @@
     </row>
     <row r="460" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A460">
-        <v>606180</v>
+        <v>656310</v>
       </c>
       <c r="B460" s="1" t="s">
         <v>1</v>
@@ -5908,7 +5908,7 @@
     </row>
     <row r="461" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A461">
-        <v>656310</v>
+        <v>416311</v>
       </c>
       <c r="B461" s="1" t="s">
         <v>1</v>
@@ -5919,7 +5919,7 @@
     </row>
     <row r="462" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A462">
-        <v>416311</v>
+        <v>406157</v>
       </c>
       <c r="B462" s="1" t="s">
         <v>1</v>
@@ -5930,7 +5930,7 @@
     </row>
     <row r="463" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A463">
-        <v>406157</v>
+        <v>416182</v>
       </c>
       <c r="B463" s="1" t="s">
         <v>1</v>
@@ -5941,18 +5941,18 @@
     </row>
     <row r="464" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A464">
-        <v>416182</v>
+        <v>406315</v>
       </c>
       <c r="B464" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C464">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="465" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A465">
-        <v>406315</v>
+        <v>406312</v>
       </c>
       <c r="B465" s="1" t="s">
         <v>1</v>
@@ -5962,19 +5962,19 @@
       </c>
     </row>
     <row r="466" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A466">
-        <v>406312</v>
+      <c r="A466" t="s">
+        <v>135</v>
       </c>
       <c r="B466" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C466">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="467" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B467" s="1" t="s">
         <v>30</v>
@@ -5988,15 +5988,15 @@
         <v>136</v>
       </c>
       <c r="B468" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C468">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="469" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B469" s="1" t="s">
         <v>1</v>
@@ -6006,14 +6006,14 @@
       </c>
     </row>
     <row r="470" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A470" t="s">
-        <v>135</v>
+      <c r="A470">
+        <v>762013</v>
       </c>
       <c r="B470" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C470">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="471" spans="1:3" x14ac:dyDescent="0.25">
@@ -6021,21 +6021,21 @@
         <v>762013</v>
       </c>
       <c r="B471" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C471">
-        <v>85</v>
+        <v>60</v>
       </c>
     </row>
     <row r="472" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A472">
-        <v>762013</v>
+      <c r="A472" t="s">
+        <v>137</v>
       </c>
       <c r="B472" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C472">
-        <v>60</v>
+        <v>90</v>
       </c>
     </row>
     <row r="473" spans="1:3" x14ac:dyDescent="0.25">
@@ -6043,21 +6043,21 @@
         <v>137</v>
       </c>
       <c r="B473" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C473">
-        <v>90</v>
+        <v>60</v>
       </c>
     </row>
     <row r="474" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B474" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C474">
-        <v>60</v>
+        <v>90</v>
       </c>
     </row>
     <row r="475" spans="1:3" x14ac:dyDescent="0.25">
@@ -6065,21 +6065,21 @@
         <v>138</v>
       </c>
       <c r="B475" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C475">
-        <v>90</v>
+        <v>60</v>
       </c>
     </row>
     <row r="476" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B476" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C476">
-        <v>60</v>
+        <v>100</v>
       </c>
     </row>
     <row r="477" spans="1:3" x14ac:dyDescent="0.25">
@@ -6087,21 +6087,21 @@
         <v>139</v>
       </c>
       <c r="B477" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C477">
-        <v>100</v>
+        <v>60</v>
       </c>
     </row>
     <row r="478" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A478" t="s">
-        <v>139</v>
+      <c r="A478">
+        <v>242020</v>
       </c>
       <c r="B478" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C478">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="479" spans="1:3" x14ac:dyDescent="0.25">
@@ -6109,21 +6109,21 @@
         <v>242020</v>
       </c>
       <c r="B479" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C479">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="480" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A480">
-        <v>242020</v>
+        <v>602010</v>
       </c>
       <c r="B480" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C480">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="481" spans="1:3" x14ac:dyDescent="0.25">
@@ -6131,21 +6131,21 @@
         <v>602010</v>
       </c>
       <c r="B481" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C481">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="482" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A482">
-        <v>602010</v>
+        <v>652010</v>
       </c>
       <c r="B482" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C482">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="483" spans="1:3" x14ac:dyDescent="0.25">
@@ -6153,37 +6153,37 @@
         <v>652010</v>
       </c>
       <c r="B483" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C483">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="484" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A484">
-        <v>652010</v>
+      <c r="A484" t="s">
+        <v>140</v>
       </c>
       <c r="B484" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C484">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="485" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A485" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B485" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C485">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="486" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A486" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B486" s="1" t="s">
         <v>1</v>
@@ -6194,7 +6194,7 @@
     </row>
     <row r="487" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A487" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B487" s="1" t="s">
         <v>1</v>
@@ -6205,29 +6205,29 @@
     </row>
     <row r="488" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B488" s="1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="C488">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="489" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A489" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B489" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C489">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="490" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A490" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B490" s="1" t="s">
         <v>56</v>
@@ -6238,7 +6238,7 @@
     </row>
     <row r="491" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A491" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B491" s="1" t="s">
         <v>56</v>
@@ -6252,26 +6252,26 @@
         <v>143</v>
       </c>
       <c r="B492" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C492">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="493" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A493" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B493" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C493">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="494" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A494" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B494" s="1" t="s">
         <v>30</v>
@@ -6282,7 +6282,7 @@
     </row>
     <row r="495" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A495" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B495" s="1" t="s">
         <v>30</v>
@@ -6293,29 +6293,29 @@
     </row>
     <row r="496" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A496" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B496" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C496">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="497" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A497" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B497" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C497">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="498" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A498" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B498" s="1" t="s">
         <v>1</v>
@@ -6326,29 +6326,29 @@
     </row>
     <row r="499" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A499" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B499" s="1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="C499">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="500" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A500" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B500" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C500">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="501" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A501" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B501" s="1" t="s">
         <v>56</v>
@@ -6362,26 +6362,26 @@
         <v>146</v>
       </c>
       <c r="B502" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C502">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="503" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A503" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B503" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C503">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="504" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A504" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B504" s="1" t="s">
         <v>30</v>
@@ -6392,13 +6392,13 @@
     </row>
     <row r="505" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A505" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B505" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C505">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="506" spans="1:3" x14ac:dyDescent="0.25">
@@ -6406,10 +6406,10 @@
         <v>147</v>
       </c>
       <c r="B506" s="1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="C506">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="507" spans="1:3" x14ac:dyDescent="0.25">
@@ -6417,18 +6417,18 @@
         <v>147</v>
       </c>
       <c r="B507" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C507">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="508" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A508" t="s">
-        <v>147</v>
+      <c r="A508">
+        <v>720004</v>
       </c>
       <c r="B508" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C508">
         <v>70</v>
@@ -6436,21 +6436,21 @@
     </row>
     <row r="509" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A509">
-        <v>720004</v>
+        <v>720003</v>
       </c>
       <c r="B509" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C509">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="510" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A510">
-        <v>720003</v>
+        <v>720004</v>
       </c>
       <c r="B510" s="1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="C510">
         <v>0</v>
@@ -6458,7 +6458,7 @@
     </row>
     <row r="511" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A511">
-        <v>720004</v>
+        <v>720003</v>
       </c>
       <c r="B511" s="1" t="s">
         <v>56</v>
@@ -6472,32 +6472,32 @@
         <v>720003</v>
       </c>
       <c r="B512" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C512">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="513" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A513">
-        <v>720003</v>
+        <v>720004</v>
       </c>
       <c r="B513" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C513">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="514" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A514">
-        <v>720004</v>
+        <v>721001</v>
       </c>
       <c r="B514" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C514">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="515" spans="1:3" x14ac:dyDescent="0.25">
@@ -6505,10 +6505,10 @@
         <v>721001</v>
       </c>
       <c r="B515" s="1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="C515">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="516" spans="1:3" x14ac:dyDescent="0.25">
@@ -6516,7 +6516,7 @@
         <v>721001</v>
       </c>
       <c r="B516" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C516">
         <v>0</v>
@@ -6524,13 +6524,13 @@
     </row>
     <row r="517" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A517">
-        <v>721001</v>
+        <v>651030</v>
       </c>
       <c r="B517" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C517">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="518" spans="1:3" x14ac:dyDescent="0.25">
@@ -6538,21 +6538,21 @@
         <v>651030</v>
       </c>
       <c r="B518" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C518">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="519" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A519">
-        <v>651030</v>
+        <v>651010</v>
       </c>
       <c r="B519" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C519">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="520" spans="1:3" x14ac:dyDescent="0.25">
@@ -6560,37 +6560,37 @@
         <v>651010</v>
       </c>
       <c r="B520" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C520">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="521" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A521">
-        <v>651010</v>
+      <c r="A521" t="s">
+        <v>148</v>
       </c>
       <c r="B521" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C521">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="522" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A522" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B522" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C522">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="523" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A523" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B523" s="1" t="s">
         <v>1</v>
@@ -6601,7 +6601,7 @@
     </row>
     <row r="524" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A524" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B524" s="1" t="s">
         <v>1</v>
@@ -6612,10 +6612,10 @@
     </row>
     <row r="525" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A525" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B525" s="1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="C525">
         <v>0</v>
@@ -6623,7 +6623,7 @@
     </row>
     <row r="526" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A526" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B526" s="1" t="s">
         <v>56</v>
@@ -6634,7 +6634,7 @@
     </row>
     <row r="527" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A527" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B527" s="1" t="s">
         <v>56</v>
@@ -6645,7 +6645,7 @@
     </row>
     <row r="528" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A528" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B528" s="1" t="s">
         <v>56</v>
@@ -6656,10 +6656,10 @@
     </row>
     <row r="529" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A529" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B529" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C529">
         <v>0</v>
@@ -6667,7 +6667,7 @@
     </row>
     <row r="530" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A530" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B530" s="1" t="s">
         <v>30</v>
@@ -6678,7 +6678,7 @@
     </row>
     <row r="531" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A531" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B531" s="1" t="s">
         <v>30</v>
@@ -6689,7 +6689,7 @@
     </row>
     <row r="532" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A532" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B532" s="1" t="s">
         <v>30</v>
@@ -6700,32 +6700,32 @@
     </row>
     <row r="533" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A533" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B533" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C533">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="534" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A534" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B534" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C534">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="535" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A535" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B535" s="1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="C535">
         <v>0</v>
@@ -6733,7 +6733,7 @@
     </row>
     <row r="536" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A536" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B536" s="1" t="s">
         <v>56</v>
@@ -6744,10 +6744,10 @@
     </row>
     <row r="537" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A537" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B537" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C537">
         <v>0</v>
@@ -6755,7 +6755,7 @@
     </row>
     <row r="538" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A538" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B538" s="1" t="s">
         <v>30</v>
@@ -6766,24 +6766,24 @@
     </row>
     <row r="539" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A539" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B539" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C539">
-        <v>0</v>
+        <v>110</v>
       </c>
     </row>
     <row r="540" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A540" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B540" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C540">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="541" spans="1:3" x14ac:dyDescent="0.25">
@@ -6791,32 +6791,32 @@
         <v>155</v>
       </c>
       <c r="B541" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C541">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="542" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A542" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B542" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C542">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="543" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A543" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B543" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C543">
-        <v>60</v>
+        <v>150</v>
       </c>
     </row>
     <row r="544" spans="1:3" x14ac:dyDescent="0.25">
@@ -6824,18 +6824,18 @@
         <v>156</v>
       </c>
       <c r="B544" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C544">
-        <v>150</v>
+        <v>110</v>
       </c>
     </row>
     <row r="545" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A545" t="s">
-        <v>156</v>
+      <c r="A545">
+        <v>721014</v>
       </c>
       <c r="B545" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C545">
         <v>110</v>
@@ -6843,24 +6843,24 @@
     </row>
     <row r="546" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A546">
-        <v>721014</v>
+        <v>721008</v>
       </c>
       <c r="B546" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C546">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="547" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A547">
-        <v>721008</v>
+        <v>721005</v>
       </c>
       <c r="B547" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C547">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="548" spans="1:3" x14ac:dyDescent="0.25">
@@ -6868,15 +6868,15 @@
         <v>721005</v>
       </c>
       <c r="B548" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C548">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="549" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A549">
-        <v>721005</v>
+        <v>721008</v>
       </c>
       <c r="B549" s="1" t="s">
         <v>1</v>
@@ -6887,24 +6887,24 @@
     </row>
     <row r="550" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A550">
-        <v>721008</v>
+        <v>721014</v>
       </c>
       <c r="B550" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C550">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="551" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A551">
-        <v>721014</v>
+      <c r="A551" t="s">
+        <v>157</v>
       </c>
       <c r="B551" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C551">
-        <v>50</v>
+        <v>110</v>
       </c>
     </row>
     <row r="552" spans="1:3" x14ac:dyDescent="0.25">
@@ -6912,32 +6912,32 @@
         <v>157</v>
       </c>
       <c r="B552" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C552">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="553" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A553" t="s">
-        <v>157</v>
+      <c r="A553">
+        <v>241040</v>
       </c>
       <c r="B553" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C553">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="554" spans="1:3" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="554" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A554">
-        <v>241040</v>
+        <v>241020</v>
       </c>
       <c r="B554" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C554">
-        <v>120</v>
+        <v>70</v>
       </c>
     </row>
     <row r="555" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6945,43 +6945,43 @@
         <v>241020</v>
       </c>
       <c r="B555" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C555">
-        <v>70</v>
+        <v>110</v>
       </c>
     </row>
     <row r="556" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A556">
-        <v>241020</v>
+        <v>241040</v>
       </c>
       <c r="B556" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C556">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="557" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A557">
-        <v>241040</v>
+        <v>601138</v>
       </c>
       <c r="B557" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C557">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="558" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A558">
-        <v>601138</v>
+        <v>601128</v>
       </c>
       <c r="B558" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C558">
-        <v>110</v>
+        <v>80</v>
       </c>
     </row>
     <row r="559" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6989,54 +6989,54 @@
         <v>601128</v>
       </c>
       <c r="B559" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C559">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="560" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A560">
-        <v>601128</v>
+        <v>601138</v>
       </c>
       <c r="B560" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C560">
-        <v>100</v>
+        <v>60</v>
       </c>
     </row>
     <row r="561" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A561">
-        <v>601138</v>
+      <c r="A561" t="s">
+        <v>158</v>
       </c>
       <c r="B561" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C561">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="562" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A562" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B562" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C562">
-        <v>120</v>
+        <v>70</v>
       </c>
     </row>
     <row r="563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A563" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B563" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C563">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7044,42 +7044,31 @@
         <v>160</v>
       </c>
       <c r="B564" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C564">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="565" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A565" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B565" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C565">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="566" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A566" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B566" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C566">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="567" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A567" t="s">
-        <v>158</v>
-      </c>
-      <c r="B567" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C567">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Profile seting time and geometry correction
</commit_message>
<xml_diff>
--- a/project/config/profile_config_file.xlsx
+++ b/project/config/profile_config_file.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsochacki\Desktop\Python\Tkinter\production-counting\project\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE0C3EA-950A-4F36-82E9-3AB764CEEB0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8801E72E-BD58-444C-80F9-D0FF16E832B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-195" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -426,9 +426,6 @@
     <t>ZF0510</t>
   </si>
   <si>
-    <t>V00219740</t>
-  </si>
-  <si>
     <t>HS9050</t>
   </si>
   <si>
@@ -553,6 +550,9 @@
   </si>
   <si>
     <t>826801</t>
+  </si>
+  <si>
+    <t>VA9740</t>
   </si>
 </sst>
 </file>
@@ -840,7 +840,7 @@
   <dimension ref="A1:C566"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" customWidth="1"/>
     <col min="2" max="2" width="20.140625" customWidth="1"/>
     <col min="3" max="3" width="12.28515625" customWidth="1"/>
     <col min="16384" max="16384" width="11.5703125" customWidth="1"/>
@@ -848,13 +848,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B1" t="s">
         <v>162</v>
       </c>
-      <c r="B1" t="s">
-        <v>163</v>
-      </c>
       <c r="C1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2289,7 +2289,7 @@
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B132" s="1" t="s">
         <v>30</v>
@@ -2311,7 +2311,7 @@
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B134" s="1" t="s">
         <v>30</v>
@@ -2322,7 +2322,7 @@
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B135" s="1" t="s">
         <v>30</v>
@@ -2333,7 +2333,7 @@
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B136" s="1" t="s">
         <v>30</v>
@@ -2344,7 +2344,7 @@
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B137" s="1" t="s">
         <v>30</v>
@@ -2355,7 +2355,7 @@
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B138" s="1" t="s">
         <v>30</v>
@@ -2366,7 +2366,7 @@
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B139" s="1" t="s">
         <v>30</v>
@@ -2377,7 +2377,7 @@
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B140" s="1" t="s">
         <v>30</v>
@@ -2388,7 +2388,7 @@
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B141" s="1" t="s">
         <v>30</v>
@@ -2399,7 +2399,7 @@
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B142" s="1" t="s">
         <v>30</v>
@@ -2410,7 +2410,7 @@
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B143" s="1" t="s">
         <v>30</v>
@@ -2421,7 +2421,7 @@
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B144" s="1" t="s">
         <v>30</v>
@@ -2432,7 +2432,7 @@
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B145" s="1" t="s">
         <v>1</v>
@@ -2443,7 +2443,7 @@
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B146" s="1" t="s">
         <v>1</v>
@@ -2454,7 +2454,7 @@
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B147" s="1" t="s">
         <v>1</v>
@@ -2465,7 +2465,7 @@
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B148" s="1" t="s">
         <v>1</v>
@@ -2476,7 +2476,7 @@
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B149" s="1" t="s">
         <v>1</v>
@@ -2487,7 +2487,7 @@
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B150" s="1" t="s">
         <v>1</v>
@@ -2498,7 +2498,7 @@
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B151" s="1" t="s">
         <v>1</v>
@@ -2509,7 +2509,7 @@
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B152" s="1" t="s">
         <v>1</v>
@@ -2520,7 +2520,7 @@
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B153" s="1" t="s">
         <v>1</v>
@@ -2531,7 +2531,7 @@
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B154" s="1" t="s">
         <v>1</v>
@@ -2542,7 +2542,7 @@
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B155" s="1" t="s">
         <v>1</v>
@@ -5842,7 +5842,7 @@
     </row>
     <row r="455" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>133</v>
+        <v>175</v>
       </c>
       <c r="B455" s="1" t="s">
         <v>1</v>
@@ -5864,7 +5864,7 @@
     </row>
     <row r="457" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B457" s="1" t="s">
         <v>1</v>
@@ -5963,7 +5963,7 @@
     </row>
     <row r="466" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B466" s="1" t="s">
         <v>30</v>
@@ -5974,7 +5974,7 @@
     </row>
     <row r="467" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B467" s="1" t="s">
         <v>30</v>
@@ -5985,7 +5985,7 @@
     </row>
     <row r="468" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B468" s="1" t="s">
         <v>1</v>
@@ -5996,7 +5996,7 @@
     </row>
     <row r="469" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B469" s="1" t="s">
         <v>1</v>
@@ -6029,7 +6029,7 @@
     </row>
     <row r="472" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B472" s="1" t="s">
         <v>30</v>
@@ -6040,7 +6040,7 @@
     </row>
     <row r="473" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B473" s="1" t="s">
         <v>1</v>
@@ -6051,7 +6051,7 @@
     </row>
     <row r="474" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B474" s="1" t="s">
         <v>30</v>
@@ -6062,7 +6062,7 @@
     </row>
     <row r="475" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B475" s="1" t="s">
         <v>1</v>
@@ -6073,7 +6073,7 @@
     </row>
     <row r="476" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B476" s="1" t="s">
         <v>30</v>
@@ -6084,7 +6084,7 @@
     </row>
     <row r="477" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B477" s="1" t="s">
         <v>1</v>
@@ -6161,7 +6161,7 @@
     </row>
     <row r="484" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A484" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B484" s="1" t="s">
         <v>1</v>
@@ -6172,7 +6172,7 @@
     </row>
     <row r="485" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A485" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B485" s="1" t="s">
         <v>1</v>
@@ -6183,7 +6183,7 @@
     </row>
     <row r="486" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A486" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B486" s="1" t="s">
         <v>1</v>
@@ -6194,7 +6194,7 @@
     </row>
     <row r="487" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A487" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B487" s="1" t="s">
         <v>1</v>
@@ -6205,7 +6205,7 @@
     </row>
     <row r="488" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B488" s="1" t="s">
         <v>56</v>
@@ -6216,7 +6216,7 @@
     </row>
     <row r="489" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A489" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B489" s="1" t="s">
         <v>56</v>
@@ -6227,7 +6227,7 @@
     </row>
     <row r="490" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A490" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B490" s="1" t="s">
         <v>56</v>
@@ -6238,7 +6238,7 @@
     </row>
     <row r="491" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A491" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B491" s="1" t="s">
         <v>56</v>
@@ -6249,7 +6249,7 @@
     </row>
     <row r="492" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A492" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B492" s="1" t="s">
         <v>30</v>
@@ -6260,7 +6260,7 @@
     </row>
     <row r="493" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A493" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B493" s="1" t="s">
         <v>30</v>
@@ -6271,7 +6271,7 @@
     </row>
     <row r="494" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A494" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B494" s="1" t="s">
         <v>30</v>
@@ -6282,7 +6282,7 @@
     </row>
     <row r="495" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A495" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B495" s="1" t="s">
         <v>30</v>
@@ -6293,7 +6293,7 @@
     </row>
     <row r="496" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A496" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B496" s="1" t="s">
         <v>1</v>
@@ -6304,7 +6304,7 @@
     </row>
     <row r="497" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A497" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B497" s="1" t="s">
         <v>1</v>
@@ -6315,7 +6315,7 @@
     </row>
     <row r="498" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A498" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B498" s="1" t="s">
         <v>1</v>
@@ -6326,7 +6326,7 @@
     </row>
     <row r="499" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A499" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B499" s="1" t="s">
         <v>56</v>
@@ -6337,7 +6337,7 @@
     </row>
     <row r="500" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A500" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B500" s="1" t="s">
         <v>56</v>
@@ -6348,7 +6348,7 @@
     </row>
     <row r="501" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A501" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B501" s="1" t="s">
         <v>56</v>
@@ -6359,7 +6359,7 @@
     </row>
     <row r="502" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A502" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B502" s="1" t="s">
         <v>30</v>
@@ -6370,7 +6370,7 @@
     </row>
     <row r="503" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A503" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B503" s="1" t="s">
         <v>30</v>
@@ -6381,7 +6381,7 @@
     </row>
     <row r="504" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A504" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B504" s="1" t="s">
         <v>30</v>
@@ -6392,7 +6392,7 @@
     </row>
     <row r="505" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A505" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B505" s="1" t="s">
         <v>1</v>
@@ -6403,7 +6403,7 @@
     </row>
     <row r="506" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A506" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B506" s="1" t="s">
         <v>56</v>
@@ -6414,7 +6414,7 @@
     </row>
     <row r="507" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A507" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B507" s="1" t="s">
         <v>30</v>
@@ -6428,7 +6428,7 @@
         <v>720004</v>
       </c>
       <c r="B508" s="1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="C508">
         <v>70</v>
@@ -6439,7 +6439,7 @@
         <v>720003</v>
       </c>
       <c r="B509" s="1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="C509">
         <v>0</v>
@@ -6450,7 +6450,7 @@
         <v>720004</v>
       </c>
       <c r="B510" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C510">
         <v>0</v>
@@ -6461,7 +6461,7 @@
         <v>720003</v>
       </c>
       <c r="B511" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C511">
         <v>0</v>
@@ -6472,10 +6472,10 @@
         <v>720003</v>
       </c>
       <c r="B512" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C512">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="513" spans="1:3" x14ac:dyDescent="0.25">
@@ -6483,7 +6483,7 @@
         <v>720004</v>
       </c>
       <c r="B513" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C513">
         <v>0</v>
@@ -6494,7 +6494,7 @@
         <v>721001</v>
       </c>
       <c r="B514" s="1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="C514">
         <v>70</v>
@@ -6505,7 +6505,7 @@
         <v>721001</v>
       </c>
       <c r="B515" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C515">
         <v>0</v>
@@ -6516,7 +6516,7 @@
         <v>721001</v>
       </c>
       <c r="B516" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C516">
         <v>0</v>
@@ -6568,7 +6568,7 @@
     </row>
     <row r="521" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A521" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B521" s="1" t="s">
         <v>1</v>
@@ -6579,7 +6579,7 @@
     </row>
     <row r="522" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A522" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B522" s="1" t="s">
         <v>1</v>
@@ -6590,7 +6590,7 @@
     </row>
     <row r="523" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A523" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B523" s="1" t="s">
         <v>1</v>
@@ -6601,7 +6601,7 @@
     </row>
     <row r="524" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A524" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B524" s="1" t="s">
         <v>1</v>
@@ -6612,7 +6612,7 @@
     </row>
     <row r="525" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A525" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B525" s="1" t="s">
         <v>56</v>
@@ -6623,7 +6623,7 @@
     </row>
     <row r="526" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A526" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B526" s="1" t="s">
         <v>56</v>
@@ -6634,7 +6634,7 @@
     </row>
     <row r="527" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A527" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B527" s="1" t="s">
         <v>56</v>
@@ -6645,7 +6645,7 @@
     </row>
     <row r="528" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A528" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B528" s="1" t="s">
         <v>56</v>
@@ -6656,7 +6656,7 @@
     </row>
     <row r="529" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A529" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B529" s="1" t="s">
         <v>30</v>
@@ -6667,7 +6667,7 @@
     </row>
     <row r="530" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A530" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B530" s="1" t="s">
         <v>30</v>
@@ -6678,7 +6678,7 @@
     </row>
     <row r="531" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A531" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B531" s="1" t="s">
         <v>30</v>
@@ -6689,7 +6689,7 @@
     </row>
     <row r="532" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A532" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B532" s="1" t="s">
         <v>30</v>
@@ -6700,7 +6700,7 @@
     </row>
     <row r="533" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A533" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B533" s="1" t="s">
         <v>1</v>
@@ -6711,7 +6711,7 @@
     </row>
     <row r="534" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A534" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B534" s="1" t="s">
         <v>1</v>
@@ -6722,7 +6722,7 @@
     </row>
     <row r="535" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A535" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B535" s="1" t="s">
         <v>56</v>
@@ -6733,7 +6733,7 @@
     </row>
     <row r="536" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A536" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B536" s="1" t="s">
         <v>56</v>
@@ -6744,7 +6744,7 @@
     </row>
     <row r="537" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A537" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B537" s="1" t="s">
         <v>30</v>
@@ -6755,7 +6755,7 @@
     </row>
     <row r="538" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A538" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B538" s="1" t="s">
         <v>30</v>
@@ -6766,7 +6766,7 @@
     </row>
     <row r="539" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A539" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B539" s="1" t="s">
         <v>30</v>
@@ -6777,7 +6777,7 @@
     </row>
     <row r="540" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A540" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B540" s="1" t="s">
         <v>30</v>
@@ -6788,7 +6788,7 @@
     </row>
     <row r="541" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A541" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B541" s="1" t="s">
         <v>1</v>
@@ -6799,7 +6799,7 @@
     </row>
     <row r="542" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A542" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B542" s="1" t="s">
         <v>1</v>
@@ -6810,7 +6810,7 @@
     </row>
     <row r="543" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A543" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B543" s="1" t="s">
         <v>30</v>
@@ -6821,7 +6821,7 @@
     </row>
     <row r="544" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A544" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B544" s="1" t="s">
         <v>1</v>
@@ -6898,7 +6898,7 @@
     </row>
     <row r="551" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A551" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B551" s="1" t="s">
         <v>30</v>
@@ -6909,7 +6909,7 @@
     </row>
     <row r="552" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A552" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B552" s="1" t="s">
         <v>1</v>
@@ -7008,7 +7008,7 @@
     </row>
     <row r="561" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A561" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B561" s="1" t="s">
         <v>30</v>
@@ -7019,7 +7019,7 @@
     </row>
     <row r="562" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A562" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B562" s="1" t="s">
         <v>30</v>
@@ -7030,7 +7030,7 @@
     </row>
     <row r="563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A563" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B563" s="1" t="s">
         <v>30</v>
@@ -7041,7 +7041,7 @@
     </row>
     <row r="564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A564" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B564" s="1" t="s">
         <v>1</v>
@@ -7052,7 +7052,7 @@
     </row>
     <row r="565" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A565" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B565" s="1" t="s">
         <v>1</v>
@@ -7063,7 +7063,7 @@
     </row>
     <row r="566" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A566" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B566" s="1" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
fix: correct the number that was entered in profile_config_file
</commit_message>
<xml_diff>
--- a/project/config/profile_config_file.xlsx
+++ b/project/config/profile_config_file.xlsx
@@ -8,15 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsochacki\Desktop\Python\Tkinter\production-counting\project\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8801E72E-BD58-444C-80F9-D0FF16E832B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1383372-D573-4D5D-A10E-784E53A926AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-195" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="profile_config" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -210,18 +221,6 @@
     <t>HS9080</t>
   </si>
   <si>
-    <t>GO 201</t>
-  </si>
-  <si>
-    <t>GO 202</t>
-  </si>
-  <si>
-    <t>GO 203</t>
-  </si>
-  <si>
-    <t>GO 209</t>
-  </si>
-  <si>
     <t>HO9820</t>
   </si>
   <si>
@@ -553,6 +552,18 @@
   </si>
   <si>
     <t>VA9740</t>
+  </si>
+  <si>
+    <t>GO2010</t>
+  </si>
+  <si>
+    <t>GO2020</t>
+  </si>
+  <si>
+    <t>GO2030</t>
+  </si>
+  <si>
+    <t>GO2090</t>
   </si>
 </sst>
 </file>
@@ -848,13 +859,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B1" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C1" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -2289,7 +2300,7 @@
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B132" s="1" t="s">
         <v>30</v>
@@ -2311,7 +2322,7 @@
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B134" s="1" t="s">
         <v>30</v>
@@ -2322,7 +2333,7 @@
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B135" s="1" t="s">
         <v>30</v>
@@ -2333,7 +2344,7 @@
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B136" s="1" t="s">
         <v>30</v>
@@ -2344,7 +2355,7 @@
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B137" s="1" t="s">
         <v>30</v>
@@ -2355,7 +2366,7 @@
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B138" s="1" t="s">
         <v>30</v>
@@ -2366,7 +2377,7 @@
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B139" s="1" t="s">
         <v>30</v>
@@ -2377,7 +2388,7 @@
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B140" s="1" t="s">
         <v>30</v>
@@ -2388,7 +2399,7 @@
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B141" s="1" t="s">
         <v>30</v>
@@ -2399,7 +2410,7 @@
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B142" s="1" t="s">
         <v>30</v>
@@ -2410,7 +2421,7 @@
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B143" s="1" t="s">
         <v>30</v>
@@ -2421,7 +2432,7 @@
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B144" s="1" t="s">
         <v>30</v>
@@ -2432,7 +2443,7 @@
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B145" s="1" t="s">
         <v>1</v>
@@ -2443,7 +2454,7 @@
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B146" s="1" t="s">
         <v>1</v>
@@ -2454,7 +2465,7 @@
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B147" s="1" t="s">
         <v>1</v>
@@ -2465,7 +2476,7 @@
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B148" s="1" t="s">
         <v>1</v>
@@ -2476,7 +2487,7 @@
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B149" s="1" t="s">
         <v>1</v>
@@ -2487,7 +2498,7 @@
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B150" s="1" t="s">
         <v>1</v>
@@ -2498,7 +2509,7 @@
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B151" s="1" t="s">
         <v>1</v>
@@ -2509,7 +2520,7 @@
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B152" s="1" t="s">
         <v>1</v>
@@ -2520,7 +2531,7 @@
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B153" s="1" t="s">
         <v>1</v>
@@ -2531,7 +2542,7 @@
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B154" s="1" t="s">
         <v>1</v>
@@ -2542,7 +2553,7 @@
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B155" s="1" t="s">
         <v>1</v>
@@ -3048,7 +3059,7 @@
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>61</v>
+        <v>172</v>
       </c>
       <c r="B201" s="1" t="s">
         <v>1</v>
@@ -3059,7 +3070,7 @@
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>62</v>
+        <v>173</v>
       </c>
       <c r="B202" s="1" t="s">
         <v>1</v>
@@ -3070,7 +3081,7 @@
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
-        <v>63</v>
+        <v>174</v>
       </c>
       <c r="B203" s="1" t="s">
         <v>1</v>
@@ -3081,7 +3092,7 @@
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>64</v>
+        <v>175</v>
       </c>
       <c r="B204" s="1" t="s">
         <v>1</v>
@@ -3202,7 +3213,7 @@
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B215" s="1" t="s">
         <v>1</v>
@@ -3213,7 +3224,7 @@
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B216" s="1" t="s">
         <v>30</v>
@@ -3224,7 +3235,7 @@
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B217" s="1" t="s">
         <v>1</v>
@@ -3279,7 +3290,7 @@
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B222" s="1" t="s">
         <v>30</v>
@@ -3301,7 +3312,7 @@
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B224" s="1" t="s">
         <v>30</v>
@@ -3323,7 +3334,7 @@
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B226" s="1" t="s">
         <v>1</v>
@@ -3345,7 +3356,7 @@
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B228" s="1" t="s">
         <v>1</v>
@@ -3356,7 +3367,7 @@
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B229" s="1" t="s">
         <v>1</v>
@@ -3367,7 +3378,7 @@
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B230" s="1" t="s">
         <v>1</v>
@@ -3455,7 +3466,7 @@
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B238" s="1" t="s">
         <v>1</v>
@@ -3466,7 +3477,7 @@
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B239" s="1" t="s">
         <v>30</v>
@@ -3477,7 +3488,7 @@
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B240" s="1" t="s">
         <v>1</v>
@@ -3488,7 +3499,7 @@
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B241" s="1" t="s">
         <v>30</v>
@@ -3499,7 +3510,7 @@
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B242" s="1" t="s">
         <v>30</v>
@@ -3510,7 +3521,7 @@
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B243" s="1" t="s">
         <v>30</v>
@@ -3521,7 +3532,7 @@
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B244" s="1" t="s">
         <v>30</v>
@@ -3620,7 +3631,7 @@
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B253" s="1" t="s">
         <v>1</v>
@@ -3631,7 +3642,7 @@
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B254" s="1" t="s">
         <v>1</v>
@@ -3642,7 +3653,7 @@
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B255" s="1" t="s">
         <v>1</v>
@@ -3653,7 +3664,7 @@
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B256" s="1" t="s">
         <v>1</v>
@@ -3664,7 +3675,7 @@
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B257" s="1" t="s">
         <v>30</v>
@@ -3675,7 +3686,7 @@
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B258" s="1" t="s">
         <v>30</v>
@@ -3686,7 +3697,7 @@
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B259" s="1" t="s">
         <v>1</v>
@@ -3697,7 +3708,7 @@
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B260" s="1" t="s">
         <v>1</v>
@@ -3708,7 +3719,7 @@
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B261" s="1" t="s">
         <v>30</v>
@@ -3719,7 +3730,7 @@
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B262" s="1" t="s">
         <v>30</v>
@@ -3730,7 +3741,7 @@
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B263" s="1" t="s">
         <v>30</v>
@@ -3763,7 +3774,7 @@
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B266" s="1" t="s">
         <v>30</v>
@@ -3774,7 +3785,7 @@
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B267" s="1" t="s">
         <v>30</v>
@@ -3807,7 +3818,7 @@
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B270" s="1" t="s">
         <v>1</v>
@@ -3818,7 +3829,7 @@
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B271" s="1" t="s">
         <v>1</v>
@@ -3851,7 +3862,7 @@
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B274" s="1" t="s">
         <v>1</v>
@@ -3862,7 +3873,7 @@
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B275" s="1" t="s">
         <v>1</v>
@@ -3873,7 +3884,7 @@
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B276" s="1" t="s">
         <v>1</v>
@@ -3884,7 +3895,7 @@
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B277" s="1" t="s">
         <v>30</v>
@@ -3917,7 +3928,7 @@
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B280" s="1" t="s">
         <v>1</v>
@@ -3942,7 +3953,7 @@
         <v>650050</v>
       </c>
       <c r="B282" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C282">
         <v>120</v>
@@ -3953,7 +3964,7 @@
         <v>650040</v>
       </c>
       <c r="B283" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C283">
         <v>90</v>
@@ -4159,7 +4170,7 @@
     </row>
     <row r="302" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B302" s="1" t="s">
         <v>30</v>
@@ -4170,7 +4181,7 @@
     </row>
     <row r="303" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B303" s="1" t="s">
         <v>1</v>
@@ -4181,7 +4192,7 @@
     </row>
     <row r="304" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B304" s="1" t="s">
         <v>30</v>
@@ -4192,7 +4203,7 @@
     </row>
     <row r="305" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B305" s="1" t="s">
         <v>1</v>
@@ -4203,10 +4214,10 @@
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B306" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C306">
         <v>120</v>
@@ -4214,10 +4225,10 @@
     </row>
     <row r="307" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B307" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C307">
         <v>0</v>
@@ -4258,7 +4269,7 @@
     </row>
     <row r="311" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B311" s="1" t="s">
         <v>30</v>
@@ -4269,7 +4280,7 @@
     </row>
     <row r="312" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B312" s="1" t="s">
         <v>1</v>
@@ -4280,7 +4291,7 @@
     </row>
     <row r="313" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B313" s="1" t="s">
         <v>30</v>
@@ -4291,7 +4302,7 @@
     </row>
     <row r="314" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B314" s="1" t="s">
         <v>1</v>
@@ -4302,7 +4313,7 @@
     </row>
     <row r="315" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B315" s="1" t="s">
         <v>1</v>
@@ -4324,7 +4335,7 @@
     </row>
     <row r="317" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B317" s="1" t="s">
         <v>30</v>
@@ -4335,7 +4346,7 @@
     </row>
     <row r="318" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B318" s="1" t="s">
         <v>30</v>
@@ -4346,7 +4357,7 @@
     </row>
     <row r="319" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B319" s="1" t="s">
         <v>30</v>
@@ -4357,7 +4368,7 @@
     </row>
     <row r="320" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B320" s="1" t="s">
         <v>30</v>
@@ -4368,7 +4379,7 @@
     </row>
     <row r="321" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B321" s="1" t="s">
         <v>30</v>
@@ -4379,7 +4390,7 @@
     </row>
     <row r="322" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B322" s="1" t="s">
         <v>30</v>
@@ -4390,7 +4401,7 @@
     </row>
     <row r="323" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B323" s="1" t="s">
         <v>30</v>
@@ -4412,7 +4423,7 @@
     </row>
     <row r="325" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B325" s="1" t="s">
         <v>30</v>
@@ -4489,7 +4500,7 @@
     </row>
     <row r="332" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B332" s="1" t="s">
         <v>1</v>
@@ -4511,7 +4522,7 @@
     </row>
     <row r="334" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="B334" s="1" t="s">
         <v>1</v>
@@ -4522,7 +4533,7 @@
     </row>
     <row r="335" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B335" s="1" t="s">
         <v>1</v>
@@ -4533,7 +4544,7 @@
     </row>
     <row r="336" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B336" s="1" t="s">
         <v>1</v>
@@ -4544,7 +4555,7 @@
     </row>
     <row r="337" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B337" s="1" t="s">
         <v>1</v>
@@ -4555,7 +4566,7 @@
     </row>
     <row r="338" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B338" s="1" t="s">
         <v>1</v>
@@ -4566,7 +4577,7 @@
     </row>
     <row r="339" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B339" s="1" t="s">
         <v>1</v>
@@ -4577,7 +4588,7 @@
     </row>
     <row r="340" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B340" s="1" t="s">
         <v>1</v>
@@ -4588,7 +4599,7 @@
     </row>
     <row r="341" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B341" s="1" t="s">
         <v>30</v>
@@ -4599,7 +4610,7 @@
     </row>
     <row r="342" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B342" s="1" t="s">
         <v>30</v>
@@ -4610,7 +4621,7 @@
     </row>
     <row r="343" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B343" s="1" t="s">
         <v>30</v>
@@ -4621,7 +4632,7 @@
     </row>
     <row r="344" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B344" s="1" t="s">
         <v>1</v>
@@ -4632,7 +4643,7 @@
     </row>
     <row r="345" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B345" s="1" t="s">
         <v>1</v>
@@ -4643,7 +4654,7 @@
     </row>
     <row r="346" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B346" s="1" t="s">
         <v>1</v>
@@ -4742,7 +4753,7 @@
     </row>
     <row r="355" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B355" s="1" t="s">
         <v>30</v>
@@ -4753,7 +4764,7 @@
     </row>
     <row r="356" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B356" s="1" t="s">
         <v>30</v>
@@ -4764,7 +4775,7 @@
     </row>
     <row r="357" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B357" s="1" t="s">
         <v>30</v>
@@ -4775,7 +4786,7 @@
     </row>
     <row r="358" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B358" s="1" t="s">
         <v>30</v>
@@ -4786,7 +4797,7 @@
     </row>
     <row r="359" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B359" s="1" t="s">
         <v>1</v>
@@ -4797,7 +4808,7 @@
     </row>
     <row r="360" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B360" s="1" t="s">
         <v>1</v>
@@ -4808,7 +4819,7 @@
     </row>
     <row r="361" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B361" s="1" t="s">
         <v>1</v>
@@ -4819,7 +4830,7 @@
     </row>
     <row r="362" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B362" s="1" t="s">
         <v>1</v>
@@ -4830,7 +4841,7 @@
     </row>
     <row r="363" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B363" s="1" t="s">
         <v>30</v>
@@ -4841,7 +4852,7 @@
     </row>
     <row r="364" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B364" s="1" t="s">
         <v>30</v>
@@ -4852,7 +4863,7 @@
     </row>
     <row r="365" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B365" s="1" t="s">
         <v>30</v>
@@ -4863,7 +4874,7 @@
     </row>
     <row r="366" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B366" s="1" t="s">
         <v>30</v>
@@ -4874,7 +4885,7 @@
     </row>
     <row r="367" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B367" s="1" t="s">
         <v>1</v>
@@ -4885,7 +4896,7 @@
     </row>
     <row r="368" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B368" s="1" t="s">
         <v>1</v>
@@ -4896,7 +4907,7 @@
     </row>
     <row r="369" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B369" s="1" t="s">
         <v>1</v>
@@ -4907,7 +4918,7 @@
     </row>
     <row r="370" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B370" s="1" t="s">
         <v>1</v>
@@ -4918,7 +4929,7 @@
     </row>
     <row r="371" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B371" s="1" t="s">
         <v>30</v>
@@ -4929,7 +4940,7 @@
     </row>
     <row r="372" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B372" s="1" t="s">
         <v>30</v>
@@ -4940,7 +4951,7 @@
     </row>
     <row r="373" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B373" s="1" t="s">
         <v>1</v>
@@ -4951,7 +4962,7 @@
     </row>
     <row r="374" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B374" s="1" t="s">
         <v>1</v>
@@ -5039,7 +5050,7 @@
     </row>
     <row r="382" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B382" s="1" t="s">
         <v>1</v>
@@ -5050,7 +5061,7 @@
     </row>
     <row r="383" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B383" s="1" t="s">
         <v>30</v>
@@ -5061,7 +5072,7 @@
     </row>
     <row r="384" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B384" s="1" t="s">
         <v>1</v>
@@ -5072,7 +5083,7 @@
     </row>
     <row r="385" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B385" s="1" t="s">
         <v>30</v>
@@ -5083,7 +5094,7 @@
     </row>
     <row r="386" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B386" s="1" t="s">
         <v>1</v>
@@ -5094,7 +5105,7 @@
     </row>
     <row r="387" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B387" s="1" t="s">
         <v>30</v>
@@ -5105,7 +5116,7 @@
     </row>
     <row r="388" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B388" s="1" t="s">
         <v>1</v>
@@ -5116,7 +5127,7 @@
     </row>
     <row r="389" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B389" s="1" t="s">
         <v>30</v>
@@ -5127,7 +5138,7 @@
     </row>
     <row r="390" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B390" s="1" t="s">
         <v>1</v>
@@ -5138,7 +5149,7 @@
     </row>
     <row r="391" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B391" s="1" t="s">
         <v>30</v>
@@ -5149,7 +5160,7 @@
     </row>
     <row r="392" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B392" s="1" t="s">
         <v>1</v>
@@ -5270,7 +5281,7 @@
     </row>
     <row r="403" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B403" s="1" t="s">
         <v>30</v>
@@ -5281,7 +5292,7 @@
     </row>
     <row r="404" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B404" s="1" t="s">
         <v>1</v>
@@ -5402,7 +5413,7 @@
     </row>
     <row r="415" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B415" s="1" t="s">
         <v>30</v>
@@ -5413,7 +5424,7 @@
     </row>
     <row r="416" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B416" s="1" t="s">
         <v>1</v>
@@ -5424,7 +5435,7 @@
     </row>
     <row r="417" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B417" s="1" t="s">
         <v>30</v>
@@ -5435,7 +5446,7 @@
     </row>
     <row r="418" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B418" s="1" t="s">
         <v>1</v>
@@ -5446,7 +5457,7 @@
     </row>
     <row r="419" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B419" s="1" t="s">
         <v>30</v>
@@ -5457,7 +5468,7 @@
     </row>
     <row r="420" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B420" s="1" t="s">
         <v>1</v>
@@ -5534,7 +5545,7 @@
     </row>
     <row r="427" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B427" s="1" t="s">
         <v>1</v>
@@ -5567,7 +5578,7 @@
     </row>
     <row r="430" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B430" s="1" t="s">
         <v>1</v>
@@ -5600,7 +5611,7 @@
     </row>
     <row r="433" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B433" s="1" t="s">
         <v>1</v>
@@ -5699,7 +5710,7 @@
     </row>
     <row r="442" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B442" s="1" t="s">
         <v>1</v>
@@ -5765,7 +5776,7 @@
     </row>
     <row r="448" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B448" s="1" t="s">
         <v>1</v>
@@ -5776,7 +5787,7 @@
     </row>
     <row r="449" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B449" s="1" t="s">
         <v>1</v>
@@ -5787,7 +5798,7 @@
     </row>
     <row r="450" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B450" s="1" t="s">
         <v>1</v>
@@ -5798,7 +5809,7 @@
     </row>
     <row r="451" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B451" s="1" t="s">
         <v>1</v>
@@ -5809,7 +5820,7 @@
     </row>
     <row r="452" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B452" s="1" t="s">
         <v>1</v>
@@ -5820,7 +5831,7 @@
     </row>
     <row r="453" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B453" s="1" t="s">
         <v>1</v>
@@ -5831,7 +5842,7 @@
     </row>
     <row r="454" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B454" s="1" t="s">
         <v>1</v>
@@ -5842,7 +5853,7 @@
     </row>
     <row r="455" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B455" s="1" t="s">
         <v>1</v>
@@ -5864,7 +5875,7 @@
     </row>
     <row r="457" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B457" s="1" t="s">
         <v>1</v>
@@ -5963,7 +5974,7 @@
     </row>
     <row r="466" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B466" s="1" t="s">
         <v>30</v>
@@ -5974,7 +5985,7 @@
     </row>
     <row r="467" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B467" s="1" t="s">
         <v>30</v>
@@ -5985,7 +5996,7 @@
     </row>
     <row r="468" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B468" s="1" t="s">
         <v>1</v>
@@ -5996,7 +6007,7 @@
     </row>
     <row r="469" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B469" s="1" t="s">
         <v>1</v>
@@ -6029,7 +6040,7 @@
     </row>
     <row r="472" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B472" s="1" t="s">
         <v>30</v>
@@ -6040,7 +6051,7 @@
     </row>
     <row r="473" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B473" s="1" t="s">
         <v>1</v>
@@ -6051,7 +6062,7 @@
     </row>
     <row r="474" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B474" s="1" t="s">
         <v>30</v>
@@ -6062,7 +6073,7 @@
     </row>
     <row r="475" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B475" s="1" t="s">
         <v>1</v>
@@ -6073,7 +6084,7 @@
     </row>
     <row r="476" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B476" s="1" t="s">
         <v>30</v>
@@ -6084,7 +6095,7 @@
     </row>
     <row r="477" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B477" s="1" t="s">
         <v>1</v>
@@ -6161,7 +6172,7 @@
     </row>
     <row r="484" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A484" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B484" s="1" t="s">
         <v>1</v>
@@ -6172,7 +6183,7 @@
     </row>
     <row r="485" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A485" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B485" s="1" t="s">
         <v>1</v>
@@ -6183,7 +6194,7 @@
     </row>
     <row r="486" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A486" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B486" s="1" t="s">
         <v>1</v>
@@ -6194,7 +6205,7 @@
     </row>
     <row r="487" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A487" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B487" s="1" t="s">
         <v>1</v>
@@ -6205,7 +6216,7 @@
     </row>
     <row r="488" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B488" s="1" t="s">
         <v>56</v>
@@ -6216,7 +6227,7 @@
     </row>
     <row r="489" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A489" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B489" s="1" t="s">
         <v>56</v>
@@ -6227,7 +6238,7 @@
     </row>
     <row r="490" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A490" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B490" s="1" t="s">
         <v>56</v>
@@ -6238,7 +6249,7 @@
     </row>
     <row r="491" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A491" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B491" s="1" t="s">
         <v>56</v>
@@ -6249,7 +6260,7 @@
     </row>
     <row r="492" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A492" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B492" s="1" t="s">
         <v>30</v>
@@ -6260,7 +6271,7 @@
     </row>
     <row r="493" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A493" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B493" s="1" t="s">
         <v>30</v>
@@ -6271,7 +6282,7 @@
     </row>
     <row r="494" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A494" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B494" s="1" t="s">
         <v>30</v>
@@ -6282,7 +6293,7 @@
     </row>
     <row r="495" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A495" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B495" s="1" t="s">
         <v>30</v>
@@ -6293,7 +6304,7 @@
     </row>
     <row r="496" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A496" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B496" s="1" t="s">
         <v>1</v>
@@ -6304,7 +6315,7 @@
     </row>
     <row r="497" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A497" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B497" s="1" t="s">
         <v>1</v>
@@ -6315,7 +6326,7 @@
     </row>
     <row r="498" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A498" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B498" s="1" t="s">
         <v>1</v>
@@ -6326,7 +6337,7 @@
     </row>
     <row r="499" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A499" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B499" s="1" t="s">
         <v>56</v>
@@ -6337,7 +6348,7 @@
     </row>
     <row r="500" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A500" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B500" s="1" t="s">
         <v>56</v>
@@ -6348,7 +6359,7 @@
     </row>
     <row r="501" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A501" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B501" s="1" t="s">
         <v>56</v>
@@ -6359,7 +6370,7 @@
     </row>
     <row r="502" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A502" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B502" s="1" t="s">
         <v>30</v>
@@ -6370,7 +6381,7 @@
     </row>
     <row r="503" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A503" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B503" s="1" t="s">
         <v>30</v>
@@ -6381,7 +6392,7 @@
     </row>
     <row r="504" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A504" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B504" s="1" t="s">
         <v>30</v>
@@ -6392,7 +6403,7 @@
     </row>
     <row r="505" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A505" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B505" s="1" t="s">
         <v>1</v>
@@ -6403,7 +6414,7 @@
     </row>
     <row r="506" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A506" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B506" s="1" t="s">
         <v>56</v>
@@ -6414,7 +6425,7 @@
     </row>
     <row r="507" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A507" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B507" s="1" t="s">
         <v>30</v>
@@ -6568,7 +6579,7 @@
     </row>
     <row r="521" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A521" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B521" s="1" t="s">
         <v>1</v>
@@ -6579,7 +6590,7 @@
     </row>
     <row r="522" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A522" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B522" s="1" t="s">
         <v>1</v>
@@ -6590,7 +6601,7 @@
     </row>
     <row r="523" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A523" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B523" s="1" t="s">
         <v>1</v>
@@ -6601,7 +6612,7 @@
     </row>
     <row r="524" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A524" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B524" s="1" t="s">
         <v>1</v>
@@ -6612,7 +6623,7 @@
     </row>
     <row r="525" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A525" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B525" s="1" t="s">
         <v>56</v>
@@ -6623,7 +6634,7 @@
     </row>
     <row r="526" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A526" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B526" s="1" t="s">
         <v>56</v>
@@ -6634,7 +6645,7 @@
     </row>
     <row r="527" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A527" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B527" s="1" t="s">
         <v>56</v>
@@ -6645,7 +6656,7 @@
     </row>
     <row r="528" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A528" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B528" s="1" t="s">
         <v>56</v>
@@ -6656,7 +6667,7 @@
     </row>
     <row r="529" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A529" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B529" s="1" t="s">
         <v>30</v>
@@ -6667,7 +6678,7 @@
     </row>
     <row r="530" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A530" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B530" s="1" t="s">
         <v>30</v>
@@ -6678,7 +6689,7 @@
     </row>
     <row r="531" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A531" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B531" s="1" t="s">
         <v>30</v>
@@ -6689,7 +6700,7 @@
     </row>
     <row r="532" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A532" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B532" s="1" t="s">
         <v>30</v>
@@ -6700,7 +6711,7 @@
     </row>
     <row r="533" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A533" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B533" s="1" t="s">
         <v>1</v>
@@ -6711,7 +6722,7 @@
     </row>
     <row r="534" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A534" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B534" s="1" t="s">
         <v>1</v>
@@ -6722,7 +6733,7 @@
     </row>
     <row r="535" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A535" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B535" s="1" t="s">
         <v>56</v>
@@ -6733,7 +6744,7 @@
     </row>
     <row r="536" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A536" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B536" s="1" t="s">
         <v>56</v>
@@ -6744,7 +6755,7 @@
     </row>
     <row r="537" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A537" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B537" s="1" t="s">
         <v>30</v>
@@ -6755,7 +6766,7 @@
     </row>
     <row r="538" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A538" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B538" s="1" t="s">
         <v>30</v>
@@ -6766,7 +6777,7 @@
     </row>
     <row r="539" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A539" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B539" s="1" t="s">
         <v>30</v>
@@ -6777,7 +6788,7 @@
     </row>
     <row r="540" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A540" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B540" s="1" t="s">
         <v>30</v>
@@ -6788,7 +6799,7 @@
     </row>
     <row r="541" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A541" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B541" s="1" t="s">
         <v>1</v>
@@ -6799,7 +6810,7 @@
     </row>
     <row r="542" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A542" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B542" s="1" t="s">
         <v>1</v>
@@ -6810,7 +6821,7 @@
     </row>
     <row r="543" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A543" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B543" s="1" t="s">
         <v>30</v>
@@ -6821,7 +6832,7 @@
     </row>
     <row r="544" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A544" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B544" s="1" t="s">
         <v>1</v>
@@ -6898,7 +6909,7 @@
     </row>
     <row r="551" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A551" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B551" s="1" t="s">
         <v>30</v>
@@ -6909,7 +6920,7 @@
     </row>
     <row r="552" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A552" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B552" s="1" t="s">
         <v>1</v>
@@ -7008,7 +7019,7 @@
     </row>
     <row r="561" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A561" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B561" s="1" t="s">
         <v>30</v>
@@ -7019,7 +7030,7 @@
     </row>
     <row r="562" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A562" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B562" s="1" t="s">
         <v>30</v>
@@ -7030,7 +7041,7 @@
     </row>
     <row r="563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A563" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B563" s="1" t="s">
         <v>30</v>
@@ -7041,7 +7052,7 @@
     </row>
     <row r="564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A564" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B564" s="1" t="s">
         <v>1</v>
@@ -7052,7 +7063,7 @@
     </row>
     <row r="565" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A565" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="B565" s="1" t="s">
         <v>1</v>
@@ -7063,7 +7074,7 @@
     </row>
     <row r="566" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A566" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B566" s="1" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
fix: correct the number that was entered in profile_config_file and missing one
</commit_message>
<xml_diff>
--- a/project/config/profile_config_file.xlsx
+++ b/project/config/profile_config_file.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsochacki\Desktop\Python\Tkinter\production-counting\project\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1383372-D573-4D5D-A10E-784E53A926AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE59DF8-0FB9-4EF2-B1EA-445367DE920A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-195" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="profile_config" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="176">
   <si>
     <t>GP8280</t>
   </si>
@@ -848,7 +848,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C566"/>
+  <dimension ref="A1:C569"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" customWidth="1"/>
@@ -3345,18 +3345,18 @@
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227">
+        <v>426100</v>
+      </c>
+      <c r="B227" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C227">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A228">
         <v>416112</v>
-      </c>
-      <c r="B227" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C227">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A228" t="s">
-        <v>63</v>
       </c>
       <c r="B228" s="1" t="s">
         <v>1</v>
@@ -3367,7 +3367,7 @@
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B229" s="1" t="s">
         <v>1</v>
@@ -3378,21 +3378,21 @@
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
+        <v>65</v>
+      </c>
+      <c r="B230" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C230">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
         <v>66</v>
       </c>
-      <c r="B230" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C230">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A231">
-        <v>406115</v>
-      </c>
       <c r="B231" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C231">
         <v>80</v>
@@ -3403,21 +3403,21 @@
         <v>406115</v>
       </c>
       <c r="B232" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C232">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233">
-        <v>666001</v>
+        <v>406115</v>
       </c>
       <c r="B233" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C233">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
@@ -3425,10 +3425,10 @@
         <v>666001</v>
       </c>
       <c r="B234" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C234">
-        <v>30</v>
+        <v>120</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
@@ -3436,54 +3436,54 @@
         <v>666001</v>
       </c>
       <c r="B235" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C235">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236">
-        <v>550801</v>
+        <v>666001</v>
       </c>
       <c r="B236" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C236">
-        <v>90</v>
+        <v>40</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237">
+        <v>550801</v>
+      </c>
+      <c r="B237" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C237">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A238">
         <v>553424</v>
       </c>
-      <c r="B237" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C237">
+      <c r="B238" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C238">
         <v>100</v>
-      </c>
-    </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A238" t="s">
-        <v>67</v>
-      </c>
-      <c r="B238" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C238">
-        <v>150</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B239" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C239">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
@@ -3491,18 +3491,18 @@
         <v>68</v>
       </c>
       <c r="B240" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C240">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B241" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C241">
         <v>90</v>
@@ -3510,40 +3510,40 @@
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B242" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C242">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B243" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C243">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
+        <v>71</v>
+      </c>
+      <c r="B244" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C244">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A245" t="s">
         <v>72</v>
-      </c>
-      <c r="B244" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C244">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A245">
-        <v>721015</v>
       </c>
       <c r="B245" s="1" t="s">
         <v>30</v>
@@ -3554,7 +3554,7 @@
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246">
-        <v>721009</v>
+        <v>721015</v>
       </c>
       <c r="B246" s="1" t="s">
         <v>30</v>
@@ -3565,7 +3565,7 @@
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247">
-        <v>341040</v>
+        <v>721009</v>
       </c>
       <c r="B247" s="1" t="s">
         <v>30</v>
@@ -3576,7 +3576,7 @@
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248">
-        <v>341030</v>
+        <v>341040</v>
       </c>
       <c r="B248" s="1" t="s">
         <v>30</v>
@@ -3590,15 +3590,15 @@
         <v>341030</v>
       </c>
       <c r="B249" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C249">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A250">
-        <v>341040</v>
+        <v>341030</v>
       </c>
       <c r="B250" s="1" t="s">
         <v>1</v>
@@ -3609,7 +3609,7 @@
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251">
-        <v>721009</v>
+        <v>341040</v>
       </c>
       <c r="B251" s="1" t="s">
         <v>1</v>
@@ -3620,7 +3620,7 @@
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252">
-        <v>721015</v>
+        <v>721009</v>
       </c>
       <c r="B252" s="1" t="s">
         <v>1</v>
@@ -3630,8 +3630,8 @@
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A253" t="s">
-        <v>72</v>
+      <c r="A253">
+        <v>721015</v>
       </c>
       <c r="B253" s="1" t="s">
         <v>1</v>
@@ -3642,7 +3642,7 @@
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B254" s="1" t="s">
         <v>1</v>
@@ -3653,46 +3653,46 @@
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B255" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C255">
-        <v>110</v>
+        <v>55</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B256" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C256">
-        <v>0</v>
+        <v>110</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B257" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C257">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B258" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C258">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
@@ -3700,37 +3700,37 @@
         <v>74</v>
       </c>
       <c r="B259" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C259">
-        <v>75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B260" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C260">
-        <v>90</v>
+        <v>75</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B261" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C261">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B262" s="1" t="s">
         <v>30</v>
@@ -3741,7 +3741,7 @@
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B263" s="1" t="s">
         <v>30</v>
@@ -3751,58 +3751,58 @@
       </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A264">
-        <v>720024</v>
+      <c r="A264" t="s">
+        <v>77</v>
       </c>
       <c r="B264" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C264">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A265">
+        <v>720024</v>
+      </c>
+      <c r="B265" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C265">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A266">
         <v>720022</v>
       </c>
-      <c r="B265" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C265">
+      <c r="B266" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C266">
         <v>70</v>
-      </c>
-    </row>
-    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A266" t="s">
-        <v>78</v>
-      </c>
-      <c r="B266" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C266">
-        <v>80</v>
       </c>
     </row>
     <row r="267" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
+        <v>78</v>
+      </c>
+      <c r="B267" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C267">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="268" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A268" t="s">
         <v>79</v>
       </c>
-      <c r="B267" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C267">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="268" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A268">
-        <v>661000</v>
-      </c>
       <c r="B268" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C268">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="269" spans="1:3" x14ac:dyDescent="0.25">
@@ -3810,15 +3810,15 @@
         <v>661000</v>
       </c>
       <c r="B269" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C269">
         <v>70</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A270" t="s">
-        <v>78</v>
+      <c r="A270">
+        <v>661000</v>
       </c>
       <c r="B270" s="1" t="s">
         <v>1</v>
@@ -3829,7 +3829,7 @@
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B271" s="1" t="s">
         <v>1</v>
@@ -3839,8 +3839,8 @@
       </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A272">
-        <v>720022</v>
+      <c r="A272" t="s">
+        <v>79</v>
       </c>
       <c r="B272" s="1" t="s">
         <v>1</v>
@@ -3851,7 +3851,7 @@
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A273">
-        <v>720024</v>
+        <v>720022</v>
       </c>
       <c r="B273" s="1" t="s">
         <v>1</v>
@@ -3861,8 +3861,8 @@
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A274" t="s">
-        <v>77</v>
+      <c r="A274">
+        <v>720024</v>
       </c>
       <c r="B274" s="1" t="s">
         <v>1</v>
@@ -3873,46 +3873,46 @@
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B275" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C275">
-        <v>110</v>
+        <v>70</v>
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B276" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C276">
-        <v>0</v>
+        <v>110</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
+        <v>75</v>
+      </c>
+      <c r="B277" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C277">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A278" t="s">
         <v>80</v>
       </c>
-      <c r="B277" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C277">
+      <c r="B278" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C278">
         <v>100</v>
-      </c>
-    </row>
-    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A278">
-        <v>416210</v>
-      </c>
-      <c r="B278" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C278">
-        <v>0</v>
       </c>
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.25">
@@ -3920,54 +3920,54 @@
         <v>416210</v>
       </c>
       <c r="B279" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C279">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="280" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A280">
+        <v>416210</v>
+      </c>
+      <c r="B280" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C280">
         <v>100</v>
       </c>
     </row>
-    <row r="280" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A280" t="s">
+    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A281" t="s">
         <v>80</v>
       </c>
-      <c r="B280" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C280">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A281">
-        <v>406210</v>
-      </c>
       <c r="B281" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C281">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A282">
-        <v>650050</v>
+        <v>406210</v>
       </c>
       <c r="B282" s="1" t="s">
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="C282">
-        <v>120</v>
+        <v>100</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283">
-        <v>650040</v>
+        <v>650050</v>
       </c>
       <c r="B283" s="1" t="s">
         <v>81</v>
       </c>
       <c r="C283">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
@@ -3975,10 +3975,10 @@
         <v>650040</v>
       </c>
       <c r="B284" s="1" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="C284">
-        <v>140</v>
+        <v>90</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
@@ -3986,21 +3986,21 @@
         <v>650040</v>
       </c>
       <c r="B285" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C285">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286">
-        <v>650050</v>
+        <v>650040</v>
       </c>
       <c r="B286" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C286">
-        <v>140</v>
+        <v>150</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.25">
@@ -4008,21 +4008,21 @@
         <v>650050</v>
       </c>
       <c r="B287" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C287">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="288" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A288">
-        <v>650020</v>
+        <v>650050</v>
       </c>
       <c r="B288" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C288">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.25">
@@ -4030,21 +4030,21 @@
         <v>650020</v>
       </c>
       <c r="B289" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C289">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A290">
-        <v>600138</v>
+        <v>650020</v>
       </c>
       <c r="B290" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C290">
-        <v>170</v>
+        <v>100</v>
       </c>
     </row>
     <row r="291" spans="1:3" x14ac:dyDescent="0.25">
@@ -4052,26 +4052,26 @@
         <v>600138</v>
       </c>
       <c r="B291" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C291">
-        <v>150</v>
+        <v>170</v>
       </c>
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A292">
-        <v>600121</v>
+        <v>600138</v>
       </c>
       <c r="B292" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C292">
-        <v>140</v>
+        <v>150</v>
       </c>
     </row>
     <row r="293" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A293">
-        <v>600127</v>
+        <v>600121</v>
       </c>
       <c r="B293" s="1" t="s">
         <v>30</v>
@@ -4085,29 +4085,29 @@
         <v>600127</v>
       </c>
       <c r="B294" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C294">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="295" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A295">
-        <v>600121</v>
+        <v>600227</v>
       </c>
       <c r="B295" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C295">
-        <v>90</v>
+        <v>140</v>
       </c>
     </row>
     <row r="296" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A296">
-        <v>600128</v>
+        <v>600227</v>
       </c>
       <c r="B296" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C296">
         <v>150</v>
@@ -4115,282 +4115,282 @@
     </row>
     <row r="297" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A297">
-        <v>600128</v>
+        <v>600127</v>
       </c>
       <c r="B297" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C297">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="298" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A298">
-        <v>650030</v>
+        <v>600121</v>
       </c>
       <c r="B298" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C298">
-        <v>170</v>
+        <v>90</v>
       </c>
     </row>
     <row r="299" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A299">
-        <v>650030</v>
+        <v>600128</v>
       </c>
       <c r="B299" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C299">
-        <v>70</v>
+        <v>150</v>
       </c>
     </row>
     <row r="300" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A300">
-        <v>660000</v>
+        <v>600128</v>
       </c>
       <c r="B300" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C300">
-        <v>120</v>
+        <v>70</v>
       </c>
     </row>
     <row r="301" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A301">
+        <v>650030</v>
+      </c>
+      <c r="B301" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C301">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A302">
+        <v>650030</v>
+      </c>
+      <c r="B302" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C302">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A303">
         <v>660000</v>
       </c>
-      <c r="B301" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C301">
+      <c r="B303" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C303">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A304">
+        <v>660000</v>
+      </c>
+      <c r="B304" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C304">
         <v>80</v>
-      </c>
-    </row>
-    <row r="302" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A302" t="s">
-        <v>82</v>
-      </c>
-      <c r="B302" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C302">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="303" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A303" t="s">
-        <v>82</v>
-      </c>
-      <c r="B303" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C303">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="304" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A304" t="s">
-        <v>83</v>
-      </c>
-      <c r="B304" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C304">
-        <v>0</v>
       </c>
     </row>
     <row r="305" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B305" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C305">
-        <v>0</v>
+        <v>110</v>
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B306" s="1" t="s">
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="C306">
-        <v>120</v>
+        <v>0</v>
       </c>
     </row>
     <row r="307" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
+        <v>83</v>
+      </c>
+      <c r="B307" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C307">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A308" t="s">
+        <v>83</v>
+      </c>
+      <c r="B308" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C308">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A309" t="s">
+        <v>83</v>
+      </c>
+      <c r="B309" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C309">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A310" t="s">
         <v>82</v>
       </c>
-      <c r="B307" s="1" t="s">
+      <c r="B310" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="C307">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="308" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A308">
+      <c r="C310">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A311">
         <v>406670</v>
       </c>
-      <c r="B308" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C308">
+      <c r="B311" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C311">
         <v>110</v>
       </c>
     </row>
-    <row r="309" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A309">
+    <row r="312" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A312">
         <v>406670</v>
       </c>
-      <c r="B309" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C309">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="310" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A310">
+      <c r="B312" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C312">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A313">
         <v>406316</v>
       </c>
-      <c r="B310" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C310">
+      <c r="B313" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C313">
         <v>120</v>
-      </c>
-    </row>
-    <row r="311" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A311" t="s">
-        <v>84</v>
-      </c>
-      <c r="B311" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C311">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="312" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A312" t="s">
-        <v>84</v>
-      </c>
-      <c r="B312" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C312">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A313" t="s">
-        <v>85</v>
-      </c>
-      <c r="B313" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C313">
-        <v>60</v>
       </c>
     </row>
     <row r="314" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B314" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C314">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="315" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B315" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C315">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A316" t="s">
+        <v>85</v>
+      </c>
+      <c r="B316" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C316">
         <v>60</v>
-      </c>
-    </row>
-    <row r="316" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A316">
-        <v>550800</v>
-      </c>
-      <c r="B316" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C316">
-        <v>80</v>
       </c>
     </row>
     <row r="317" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B317" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C317">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="318" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B318" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C318">
         <v>60</v>
       </c>
     </row>
     <row r="319" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A319" t="s">
-        <v>89</v>
+      <c r="A319">
+        <v>550800</v>
       </c>
       <c r="B319" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C319">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="320" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B320" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C320">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="321" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B321" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C321">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="322" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B322" s="1" t="s">
         <v>30</v>
@@ -4401,7 +4401,7 @@
     </row>
     <row r="323" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B323" s="1" t="s">
         <v>30</v>
@@ -4411,66 +4411,66 @@
       </c>
     </row>
     <row r="324" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A324">
-        <v>720023</v>
+      <c r="A324" t="s">
+        <v>91</v>
       </c>
       <c r="B324" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C324">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="325" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B325" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C325">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="326" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A326">
-        <v>240040</v>
+      <c r="A326" t="s">
+        <v>93</v>
       </c>
       <c r="B326" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C326">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="327" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A327">
-        <v>240030</v>
+        <v>720023</v>
       </c>
       <c r="B327" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C327">
-        <v>50</v>
+        <v>80</v>
       </c>
     </row>
     <row r="328" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A328">
-        <v>240020</v>
+      <c r="A328" t="s">
+        <v>94</v>
       </c>
       <c r="B328" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C328">
-        <v>50</v>
+        <v>70</v>
       </c>
     </row>
     <row r="329" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A329">
-        <v>240020</v>
+        <v>240040</v>
       </c>
       <c r="B329" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C329">
         <v>60</v>
@@ -4481,7 +4481,7 @@
         <v>240030</v>
       </c>
       <c r="B330" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C330">
         <v>50</v>
@@ -4489,84 +4489,84 @@
     </row>
     <row r="331" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A331">
-        <v>240040</v>
+        <v>240020</v>
       </c>
       <c r="B331" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C331">
         <v>50</v>
       </c>
     </row>
     <row r="332" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A332" t="s">
-        <v>94</v>
+      <c r="A332">
+        <v>240020</v>
       </c>
       <c r="B332" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C332">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="333" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A333">
-        <v>720023</v>
+        <v>240030</v>
       </c>
       <c r="B333" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C333">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="334" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A334" t="s">
-        <v>93</v>
+      <c r="A334">
+        <v>240040</v>
       </c>
       <c r="B334" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C334">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="335" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B335" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C335">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="336" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A336" t="s">
-        <v>91</v>
+      <c r="A336">
+        <v>720023</v>
       </c>
       <c r="B336" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C336">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="337" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B337" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C337">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="338" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B338" s="1" t="s">
         <v>1</v>
@@ -4577,7 +4577,7 @@
     </row>
     <row r="339" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B339" s="1" t="s">
         <v>1</v>
@@ -4588,57 +4588,57 @@
     </row>
     <row r="340" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B340" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C340">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="341" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B341" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C341">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="342" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="B342" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C342">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="343" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="B343" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C343">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="344" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B344" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C344">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="345" spans="1:3" x14ac:dyDescent="0.25">
@@ -4646,76 +4646,76 @@
         <v>96</v>
       </c>
       <c r="B345" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C345">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="346" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
+        <v>97</v>
+      </c>
+      <c r="B346" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C346">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="347" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A347" t="s">
+        <v>97</v>
+      </c>
+      <c r="B347" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C347">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="348" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A348" t="s">
+        <v>96</v>
+      </c>
+      <c r="B348" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C348">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="349" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A349" t="s">
         <v>95</v>
       </c>
-      <c r="B346" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C346">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="347" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A347">
-        <v>722010</v>
-      </c>
-      <c r="B347" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C347">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="348" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A348">
-        <v>722005</v>
-      </c>
-      <c r="B348" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C348">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="349" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A349">
-        <v>722006</v>
-      </c>
       <c r="B349" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C349">
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="350" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A350">
-        <v>722000</v>
+        <v>722010</v>
       </c>
       <c r="B350" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C350">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="351" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A351">
-        <v>722000</v>
+        <v>722005</v>
       </c>
       <c r="B351" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C351">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="352" spans="1:3" x14ac:dyDescent="0.25">
@@ -4723,7 +4723,7 @@
         <v>722006</v>
       </c>
       <c r="B352" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C352">
         <v>0</v>
@@ -4731,79 +4731,79 @@
     </row>
     <row r="353" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A353">
-        <v>722005</v>
+        <v>722000</v>
       </c>
       <c r="B353" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C353">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="354" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A354">
+        <v>722000</v>
+      </c>
+      <c r="B354" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C354">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="355" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A355">
+        <v>722006</v>
+      </c>
+      <c r="B355" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C355">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="356" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A356">
+        <v>722005</v>
+      </c>
+      <c r="B356" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C356">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="357" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A357">
         <v>722010</v>
       </c>
-      <c r="B354" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C354">
+      <c r="B357" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C357">
         <v>50</v>
-      </c>
-    </row>
-    <row r="355" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A355" t="s">
-        <v>98</v>
-      </c>
-      <c r="B355" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C355">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="356" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A356" t="s">
-        <v>99</v>
-      </c>
-      <c r="B356" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C356">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="357" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A357" t="s">
-        <v>100</v>
-      </c>
-      <c r="B357" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C357">
-        <v>0</v>
       </c>
     </row>
     <row r="358" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B358" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C358">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="359" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B359" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C359">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="360" spans="1:3" x14ac:dyDescent="0.25">
@@ -4811,62 +4811,62 @@
         <v>100</v>
       </c>
       <c r="B360" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C360">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="361" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B361" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C361">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="362" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B362" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C362">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="363" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B363" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C363">
-        <v>100</v>
+        <v>50</v>
       </c>
     </row>
     <row r="364" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B364" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C364">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="365" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B365" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C365">
         <v>0</v>
@@ -4874,24 +4874,24 @@
     </row>
     <row r="366" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B366" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C366">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="367" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B367" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C367">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="368" spans="1:3" x14ac:dyDescent="0.25">
@@ -4899,7 +4899,7 @@
         <v>104</v>
       </c>
       <c r="B368" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C368">
         <v>0</v>
@@ -4907,10 +4907,10 @@
     </row>
     <row r="369" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B369" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C369">
         <v>0</v>
@@ -4918,7 +4918,7 @@
     </row>
     <row r="370" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B370" s="1" t="s">
         <v>1</v>
@@ -4929,29 +4929,29 @@
     </row>
     <row r="371" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B371" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C371">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="372" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B372" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C372">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="373" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B373" s="1" t="s">
         <v>1</v>
@@ -4965,59 +4965,59 @@
         <v>106</v>
       </c>
       <c r="B374" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C374">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="375" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A375" t="s">
+        <v>107</v>
+      </c>
+      <c r="B375" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C375">
         <v>60</v>
       </c>
     </row>
-    <row r="375" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A375">
-        <v>406010</v>
-      </c>
-      <c r="B375" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C375">
-        <v>120</v>
-      </c>
-    </row>
     <row r="376" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A376">
-        <v>406321</v>
+      <c r="A376" t="s">
+        <v>107</v>
       </c>
       <c r="B376" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C376">
-        <v>150</v>
+        <v>70</v>
       </c>
     </row>
     <row r="377" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A377">
-        <v>406660</v>
+      <c r="A377" t="s">
+        <v>106</v>
       </c>
       <c r="B377" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C377">
-        <v>120</v>
+        <v>60</v>
       </c>
     </row>
     <row r="378" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A378">
-        <v>406329</v>
+        <v>406010</v>
       </c>
       <c r="B378" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C378">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="379" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A379">
-        <v>406325</v>
+        <v>406321</v>
       </c>
       <c r="B379" s="1" t="s">
         <v>1</v>
@@ -5028,10 +5028,10 @@
     </row>
     <row r="380" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A380">
-        <v>416240</v>
+        <v>406660</v>
       </c>
       <c r="B380" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C380">
         <v>120</v>
@@ -5039,54 +5039,54 @@
     </row>
     <row r="381" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A381">
+        <v>406329</v>
+      </c>
+      <c r="B381" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C381">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="382" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A382">
+        <v>406325</v>
+      </c>
+      <c r="B382" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C382">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="383" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A383">
         <v>416240</v>
       </c>
-      <c r="B381" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C381">
+      <c r="B383" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C383">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="384" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A384">
+        <v>416240</v>
+      </c>
+      <c r="B384" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C384">
         <v>100</v>
-      </c>
-    </row>
-    <row r="382" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A382" t="s">
-        <v>108</v>
-      </c>
-      <c r="B382" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C382">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="383" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A383" t="s">
-        <v>109</v>
-      </c>
-      <c r="B383" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C383">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="384" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A384" t="s">
-        <v>109</v>
-      </c>
-      <c r="B384" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C384">
-        <v>120</v>
       </c>
     </row>
     <row r="385" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B385" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C385">
         <v>100</v>
@@ -5094,10 +5094,10 @@
     </row>
     <row r="386" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B386" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C386">
         <v>100</v>
@@ -5105,120 +5105,120 @@
     </row>
     <row r="387" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B387" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C387">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="388" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B388" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C388">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="389" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B389" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C389">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="390" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B390" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C390">
-        <v>130</v>
+        <v>100</v>
       </c>
     </row>
     <row r="391" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B391" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C391">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="392" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
+        <v>112</v>
+      </c>
+      <c r="B392" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C392">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="393" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A393" t="s">
+        <v>112</v>
+      </c>
+      <c r="B393" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C393">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="394" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A394" t="s">
         <v>113</v>
       </c>
-      <c r="B392" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C392">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="393" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A393">
-        <v>242320</v>
-      </c>
-      <c r="B393" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C393">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="394" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A394">
-        <v>242320</v>
-      </c>
       <c r="B394" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C394">
         <v>100</v>
       </c>
     </row>
     <row r="395" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A395">
-        <v>651050</v>
+      <c r="A395" t="s">
+        <v>113</v>
       </c>
       <c r="B395" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C395">
-        <v>110</v>
+        <v>130</v>
       </c>
     </row>
     <row r="396" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A396">
-        <v>651050</v>
+        <v>242320</v>
       </c>
       <c r="B396" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C396">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="397" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A397">
-        <v>730010</v>
+        <v>242320</v>
       </c>
       <c r="B397" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C397">
         <v>100</v>
@@ -5226,241 +5226,241 @@
     </row>
     <row r="398" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A398">
-        <v>730010</v>
+        <v>651050</v>
       </c>
       <c r="B398" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C398">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="399" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A399">
-        <v>731020</v>
+        <v>651050</v>
       </c>
       <c r="B399" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C399">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="400" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A400">
-        <v>731020</v>
+        <v>730010</v>
       </c>
       <c r="B400" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C400">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="401" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A401">
-        <v>476273</v>
+        <v>730010</v>
       </c>
       <c r="B401" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C401">
-        <v>60</v>
+        <v>100</v>
       </c>
     </row>
     <row r="402" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A402">
+        <v>731020</v>
+      </c>
+      <c r="B402" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C402">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="403" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A403">
+        <v>731020</v>
+      </c>
+      <c r="B403" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C403">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="404" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A404">
         <v>476273</v>
       </c>
-      <c r="B402" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C402">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="403" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A403" t="s">
-        <v>114</v>
-      </c>
-      <c r="B403" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C403">
+      <c r="B404" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C404">
         <v>60</v>
-      </c>
-    </row>
-    <row r="404" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A404" t="s">
-        <v>114</v>
-      </c>
-      <c r="B404" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C404">
-        <v>0</v>
       </c>
     </row>
     <row r="405" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A405">
-        <v>466009</v>
+        <v>476273</v>
       </c>
       <c r="B405" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C405">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="406" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A406" t="s">
+        <v>114</v>
+      </c>
+      <c r="B406" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C406">
         <v>60</v>
       </c>
     </row>
-    <row r="406" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A406">
-        <v>466009</v>
-      </c>
-      <c r="B406" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C406">
-        <v>0</v>
-      </c>
-    </row>
     <row r="407" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A407">
-        <v>416273</v>
+      <c r="A407" t="s">
+        <v>114</v>
       </c>
       <c r="B407" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C407">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="408" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A408">
-        <v>416273</v>
+        <v>466009</v>
       </c>
       <c r="B408" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C408">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="409" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A409">
-        <v>466023</v>
+        <v>466009</v>
       </c>
       <c r="B409" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C409">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="410" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A410">
-        <v>466023</v>
+        <v>416273</v>
       </c>
       <c r="B410" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C410">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="411" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A411">
-        <v>426200</v>
+        <v>416273</v>
       </c>
       <c r="B411" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C411">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="412" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A412">
-        <v>426200</v>
+        <v>466023</v>
       </c>
       <c r="B412" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C412">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="413" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A413">
-        <v>406272</v>
+        <v>466023</v>
       </c>
       <c r="B413" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C413">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="414" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A414">
+        <v>426200</v>
+      </c>
+      <c r="B414" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C414">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="415" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A415">
+        <v>426200</v>
+      </c>
+      <c r="B415" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C415">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="416" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A416">
         <v>406272</v>
       </c>
-      <c r="B414" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C414">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="415" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A415" t="s">
-        <v>115</v>
-      </c>
-      <c r="B415" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C415">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="416" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A416" t="s">
-        <v>115</v>
-      </c>
       <c r="B416" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C416">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="417" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A417" t="s">
-        <v>116</v>
+      <c r="A417">
+        <v>406272</v>
       </c>
       <c r="B417" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C417">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="418" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B418" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C418">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="419" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B419" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C419">
         <v>80</v>
@@ -5468,172 +5468,172 @@
     </row>
     <row r="420" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
+        <v>116</v>
+      </c>
+      <c r="B420" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C420">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="421" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A421" t="s">
+        <v>116</v>
+      </c>
+      <c r="B421" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C421">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="422" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A422" t="s">
         <v>117</v>
       </c>
-      <c r="B420" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C420">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="421" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A421">
-        <v>416338</v>
-      </c>
-      <c r="B421" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C421">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="422" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A422">
-        <v>416331</v>
-      </c>
       <c r="B422" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C422">
-        <v>200</v>
+        <v>80</v>
       </c>
     </row>
     <row r="423" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A423">
-        <v>416065</v>
+      <c r="A423" t="s">
+        <v>117</v>
       </c>
       <c r="B423" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C423">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="424" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A424">
-        <v>416067</v>
+        <v>416338</v>
       </c>
       <c r="B424" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C424">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="425" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A425">
-        <v>416086</v>
+        <v>416331</v>
       </c>
       <c r="B425" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C425">
-        <v>90</v>
+        <v>200</v>
       </c>
     </row>
     <row r="426" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A426">
-        <v>416096</v>
+        <v>416065</v>
       </c>
       <c r="B426" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C426">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="427" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A427">
+        <v>416067</v>
+      </c>
+      <c r="B427" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C427">
         <v>120</v>
-      </c>
-    </row>
-    <row r="427" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A427" t="s">
-        <v>118</v>
-      </c>
-      <c r="B427" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C427">
-        <v>90</v>
       </c>
     </row>
     <row r="428" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A428">
-        <v>666003</v>
+        <v>416086</v>
       </c>
       <c r="B428" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C428">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="429" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A429">
-        <v>666002</v>
+        <v>416096</v>
       </c>
       <c r="B429" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C429">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="430" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A430" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B430" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C430">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="431" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A431">
-        <v>416070</v>
+        <v>666003</v>
       </c>
       <c r="B431" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C431">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="432" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A432">
-        <v>416069</v>
+        <v>666002</v>
       </c>
       <c r="B432" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C432">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="433" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B433" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C433">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="434" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A434">
-        <v>406340</v>
+        <v>416070</v>
       </c>
       <c r="B434" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C434">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="435" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A435">
-        <v>416301</v>
+        <v>416069</v>
       </c>
       <c r="B435" s="1" t="s">
         <v>1</v>
@@ -5643,19 +5643,19 @@
       </c>
     </row>
     <row r="436" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A436">
-        <v>416119</v>
+      <c r="A436" t="s">
+        <v>120</v>
       </c>
       <c r="B436" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C436">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="437" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A437">
-        <v>406081</v>
+        <v>406340</v>
       </c>
       <c r="B437" s="1" t="s">
         <v>1</v>
@@ -5666,62 +5666,62 @@
     </row>
     <row r="438" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A438">
-        <v>416068</v>
+        <v>416301</v>
       </c>
       <c r="B438" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C438">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="439" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A439">
-        <v>416068</v>
+        <v>416119</v>
       </c>
       <c r="B439" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C439">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="440" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A440">
-        <v>736315</v>
+        <v>406081</v>
       </c>
       <c r="B440" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C440">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="441" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A441">
-        <v>736334</v>
+        <v>416068</v>
       </c>
       <c r="B441" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C441">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="442" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A442" t="s">
-        <v>121</v>
+      <c r="A442">
+        <v>416068</v>
       </c>
       <c r="B442" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C442">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="443" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A443">
-        <v>406307</v>
+        <v>736315</v>
       </c>
       <c r="B443" s="1" t="s">
         <v>1</v>
@@ -5732,7 +5732,7 @@
     </row>
     <row r="444" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A444">
-        <v>466400</v>
+        <v>736334</v>
       </c>
       <c r="B444" s="1" t="s">
         <v>1</v>
@@ -5742,118 +5742,118 @@
       </c>
     </row>
     <row r="445" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A445">
-        <v>416139</v>
+      <c r="A445" t="s">
+        <v>121</v>
       </c>
       <c r="B445" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C445">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="446" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A446">
-        <v>416139</v>
+        <v>406307</v>
       </c>
       <c r="B446" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C446">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="447" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A447">
+        <v>466400</v>
+      </c>
+      <c r="B447" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C447">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="448" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A448">
+        <v>416139</v>
+      </c>
+      <c r="B448" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C448">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="449" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A449">
+        <v>416139</v>
+      </c>
+      <c r="B449" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C449">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="450" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A450">
         <v>416148</v>
       </c>
-      <c r="B447" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C447">
+      <c r="B450" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C450">
         <v>80</v>
-      </c>
-    </row>
-    <row r="448" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A448" t="s">
-        <v>122</v>
-      </c>
-      <c r="B448" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C448">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="449" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A449" t="s">
-        <v>123</v>
-      </c>
-      <c r="B449" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C449">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="450" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A450" t="s">
-        <v>124</v>
-      </c>
-      <c r="B450" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C450">
-        <v>100</v>
       </c>
     </row>
     <row r="451" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B451" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C451">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="452" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B452" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C452">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="453" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B453" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C453">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="454" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B454" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C454">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="455" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>171</v>
+        <v>126</v>
       </c>
       <c r="B455" s="1" t="s">
         <v>1</v>
@@ -5863,8 +5863,8 @@
       </c>
     </row>
     <row r="456" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A456">
-        <v>406310</v>
+      <c r="A456" t="s">
+        <v>127</v>
       </c>
       <c r="B456" s="1" t="s">
         <v>1</v>
@@ -5875,7 +5875,7 @@
     </row>
     <row r="457" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B457" s="1" t="s">
         <v>1</v>
@@ -5885,8 +5885,8 @@
       </c>
     </row>
     <row r="458" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A458">
-        <v>416180</v>
+      <c r="A458" t="s">
+        <v>171</v>
       </c>
       <c r="B458" s="1" t="s">
         <v>1</v>
@@ -5897,18 +5897,18 @@
     </row>
     <row r="459" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A459">
-        <v>606180</v>
+        <v>406310</v>
       </c>
       <c r="B459" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C459">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="460" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A460">
-        <v>656310</v>
+      <c r="A460" t="s">
+        <v>129</v>
       </c>
       <c r="B460" s="1" t="s">
         <v>1</v>
@@ -5919,7 +5919,7 @@
     </row>
     <row r="461" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A461">
-        <v>416311</v>
+        <v>416180</v>
       </c>
       <c r="B461" s="1" t="s">
         <v>1</v>
@@ -5930,7 +5930,7 @@
     </row>
     <row r="462" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A462">
-        <v>406157</v>
+        <v>606180</v>
       </c>
       <c r="B462" s="1" t="s">
         <v>1</v>
@@ -5941,7 +5941,7 @@
     </row>
     <row r="463" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A463">
-        <v>416182</v>
+        <v>656310</v>
       </c>
       <c r="B463" s="1" t="s">
         <v>1</v>
@@ -5952,57 +5952,57 @@
     </row>
     <row r="464" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A464">
-        <v>406315</v>
+        <v>416311</v>
       </c>
       <c r="B464" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C464">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="465" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A465">
+        <v>406157</v>
+      </c>
+      <c r="B465" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C465">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="466" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A466">
+        <v>416182</v>
+      </c>
+      <c r="B466" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C466">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="467" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A467">
+        <v>406315</v>
+      </c>
+      <c r="B467" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C467">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="468" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A468">
         <v>406312</v>
       </c>
-      <c r="B465" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C465">
+      <c r="B468" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C468">
         <v>100</v>
-      </c>
-    </row>
-    <row r="466" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A466" t="s">
-        <v>130</v>
-      </c>
-      <c r="B466" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C466">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="467" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A467" t="s">
-        <v>131</v>
-      </c>
-      <c r="B467" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C467">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="468" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A468" t="s">
-        <v>131</v>
-      </c>
-      <c r="B468" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C468">
-        <v>70</v>
       </c>
     </row>
     <row r="469" spans="1:3" x14ac:dyDescent="0.25">
@@ -6010,227 +6010,227 @@
         <v>130</v>
       </c>
       <c r="B469" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C469">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="470" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A470" t="s">
+        <v>131</v>
+      </c>
+      <c r="B470" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C470">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="471" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A471" t="s">
+        <v>131</v>
+      </c>
+      <c r="B471" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C471">
         <v>70</v>
-      </c>
-    </row>
-    <row r="470" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A470">
-        <v>762013</v>
-      </c>
-      <c r="B470" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C470">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="471" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A471">
-        <v>762013</v>
-      </c>
-      <c r="B471" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C471">
-        <v>60</v>
       </c>
     </row>
     <row r="472" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B472" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C472">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="473" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A473" t="s">
-        <v>132</v>
+      <c r="A473">
+        <v>762013</v>
       </c>
       <c r="B473" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C473">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="474" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A474">
+        <v>762013</v>
+      </c>
+      <c r="B474" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C474">
         <v>60</v>
-      </c>
-    </row>
-    <row r="474" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A474" t="s">
-        <v>133</v>
-      </c>
-      <c r="B474" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C474">
-        <v>90</v>
       </c>
     </row>
     <row r="475" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B475" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C475">
-        <v>60</v>
+        <v>90</v>
       </c>
     </row>
     <row r="476" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B476" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C476">
-        <v>100</v>
+        <v>60</v>
       </c>
     </row>
     <row r="477" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
+        <v>133</v>
+      </c>
+      <c r="B477" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C477">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="478" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A478" t="s">
+        <v>133</v>
+      </c>
+      <c r="B478" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C478">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="479" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A479" t="s">
         <v>134</v>
       </c>
-      <c r="B477" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C477">
+      <c r="B479" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C479">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="480" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A480" t="s">
+        <v>134</v>
+      </c>
+      <c r="B480" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C480">
         <v>60</v>
-      </c>
-    </row>
-    <row r="478" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A478">
-        <v>242020</v>
-      </c>
-      <c r="B478" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C478">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="479" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A479">
-        <v>242020</v>
-      </c>
-      <c r="B479" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C479">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="480" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A480">
-        <v>602010</v>
-      </c>
-      <c r="B480" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C480">
-        <v>80</v>
       </c>
     </row>
     <row r="481" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A481">
-        <v>602010</v>
+        <v>242020</v>
       </c>
       <c r="B481" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C481">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="482" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A482">
-        <v>652010</v>
+        <v>242020</v>
       </c>
       <c r="B482" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C482">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="483" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A483">
+        <v>602010</v>
+      </c>
+      <c r="B483" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C483">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="484" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A484">
+        <v>602010</v>
+      </c>
+      <c r="B484" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C484">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="485" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A485">
         <v>652010</v>
       </c>
-      <c r="B483" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C483">
+      <c r="B485" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C485">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="486" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A486">
+        <v>652010</v>
+      </c>
+      <c r="B486" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C486">
         <v>60</v>
-      </c>
-    </row>
-    <row r="484" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A484" t="s">
-        <v>135</v>
-      </c>
-      <c r="B484" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C484">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="485" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A485" t="s">
-        <v>136</v>
-      </c>
-      <c r="B485" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C485">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="486" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A486" t="s">
-        <v>137</v>
-      </c>
-      <c r="B486" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C486">
-        <v>0</v>
       </c>
     </row>
     <row r="487" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A487" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B487" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C487">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="488" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B488" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C488">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="489" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A489" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B489" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C489">
         <v>0</v>
@@ -6238,10 +6238,10 @@
     </row>
     <row r="490" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A490" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B490" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C490">
         <v>0</v>
@@ -6249,24 +6249,24 @@
     </row>
     <row r="491" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A491" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B491" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C491">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="492" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A492" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B492" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C492">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="493" spans="1:3" x14ac:dyDescent="0.25">
@@ -6274,7 +6274,7 @@
         <v>137</v>
       </c>
       <c r="B493" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C493">
         <v>0</v>
@@ -6282,10 +6282,10 @@
     </row>
     <row r="494" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A494" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B494" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C494">
         <v>0</v>
@@ -6293,32 +6293,32 @@
     </row>
     <row r="495" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A495" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B495" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C495">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="496" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A496" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B496" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C496">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="497" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A497" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B497" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C497">
         <v>0</v>
@@ -6326,10 +6326,10 @@
     </row>
     <row r="498" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A498" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="B498" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C498">
         <v>0</v>
@@ -6340,7 +6340,7 @@
         <v>139</v>
       </c>
       <c r="B499" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C499">
         <v>70</v>
@@ -6351,7 +6351,7 @@
         <v>140</v>
       </c>
       <c r="B500" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C500">
         <v>0</v>
@@ -6362,7 +6362,7 @@
         <v>141</v>
       </c>
       <c r="B501" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C501">
         <v>0</v>
@@ -6370,10 +6370,10 @@
     </row>
     <row r="502" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A502" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B502" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C502">
         <v>70</v>
@@ -6384,7 +6384,7 @@
         <v>140</v>
       </c>
       <c r="B503" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C503">
         <v>0</v>
@@ -6392,10 +6392,10 @@
     </row>
     <row r="504" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A504" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B504" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C504">
         <v>0</v>
@@ -6403,10 +6403,10 @@
     </row>
     <row r="505" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A505" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B505" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C505">
         <v>70</v>
@@ -6414,10 +6414,10 @@
     </row>
     <row r="506" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A506" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B506" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C506">
         <v>0</v>
@@ -6425,29 +6425,29 @@
     </row>
     <row r="507" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A507" t="s">
+        <v>139</v>
+      </c>
+      <c r="B507" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C507">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="508" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A508" t="s">
         <v>142</v>
       </c>
-      <c r="B507" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C507">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="508" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A508">
-        <v>720004</v>
-      </c>
       <c r="B508" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C508">
         <v>70</v>
       </c>
     </row>
     <row r="509" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A509">
-        <v>720003</v>
+      <c r="A509" t="s">
+        <v>142</v>
       </c>
       <c r="B509" s="1" t="s">
         <v>56</v>
@@ -6457,25 +6457,25 @@
       </c>
     </row>
     <row r="510" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A510">
-        <v>720004</v>
+      <c r="A510" t="s">
+        <v>142</v>
       </c>
       <c r="B510" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C510">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="511" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A511">
-        <v>720003</v>
+        <v>720004</v>
       </c>
       <c r="B511" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C511">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="512" spans="1:3" x14ac:dyDescent="0.25">
@@ -6483,7 +6483,7 @@
         <v>720003</v>
       </c>
       <c r="B512" s="1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="C512">
         <v>0</v>
@@ -6494,7 +6494,7 @@
         <v>720004</v>
       </c>
       <c r="B513" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C513">
         <v>0</v>
@@ -6502,21 +6502,21 @@
     </row>
     <row r="514" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A514">
-        <v>721001</v>
+        <v>720003</v>
       </c>
       <c r="B514" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C514">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="515" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A515">
-        <v>721001</v>
+        <v>720003</v>
       </c>
       <c r="B515" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C515">
         <v>0</v>
@@ -6524,7 +6524,7 @@
     </row>
     <row r="516" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A516">
-        <v>721001</v>
+        <v>720004</v>
       </c>
       <c r="B516" s="1" t="s">
         <v>1</v>
@@ -6535,7 +6535,7 @@
     </row>
     <row r="517" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A517">
-        <v>651030</v>
+        <v>721001</v>
       </c>
       <c r="B517" s="1" t="s">
         <v>56</v>
@@ -6546,7 +6546,7 @@
     </row>
     <row r="518" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A518">
-        <v>651030</v>
+        <v>721001</v>
       </c>
       <c r="B518" s="1" t="s">
         <v>30</v>
@@ -6557,54 +6557,54 @@
     </row>
     <row r="519" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A519">
-        <v>651010</v>
+        <v>721001</v>
       </c>
       <c r="B519" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C519">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="520" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A520">
+        <v>651030</v>
+      </c>
+      <c r="B520" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C520">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="521" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A521">
+        <v>651030</v>
+      </c>
+      <c r="B521" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C521">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="522" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A522">
         <v>651010</v>
       </c>
-      <c r="B520" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C520">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="521" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A521" t="s">
-        <v>143</v>
-      </c>
-      <c r="B521" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C521">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="522" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A522" t="s">
-        <v>144</v>
-      </c>
       <c r="B522" s="1" t="s">
-        <v>1</v>
+        <v>56</v>
       </c>
       <c r="C522">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="523" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A523" t="s">
-        <v>145</v>
+      <c r="A523">
+        <v>651010</v>
       </c>
       <c r="B523" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C523">
         <v>0</v>
@@ -6612,21 +6612,21 @@
     </row>
     <row r="524" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A524" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B524" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C524">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="525" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A525" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B525" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C525">
         <v>0</v>
@@ -6634,10 +6634,10 @@
     </row>
     <row r="526" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A526" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B526" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C526">
         <v>0</v>
@@ -6645,10 +6645,10 @@
     </row>
     <row r="527" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A527" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B527" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C527">
         <v>0</v>
@@ -6656,7 +6656,7 @@
     </row>
     <row r="528" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A528" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B528" s="1" t="s">
         <v>56</v>
@@ -6667,10 +6667,10 @@
     </row>
     <row r="529" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A529" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B529" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C529">
         <v>0</v>
@@ -6678,10 +6678,10 @@
     </row>
     <row r="530" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A530" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B530" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C530">
         <v>0</v>
@@ -6689,10 +6689,10 @@
     </row>
     <row r="531" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A531" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B531" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C531">
         <v>0</v>
@@ -6700,7 +6700,7 @@
     </row>
     <row r="532" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A532" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B532" s="1" t="s">
         <v>30</v>
@@ -6711,21 +6711,21 @@
     </row>
     <row r="533" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A533" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B533" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C533">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="534" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A534" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B534" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C534">
         <v>0</v>
@@ -6733,10 +6733,10 @@
     </row>
     <row r="535" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A535" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B535" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C535">
         <v>0</v>
@@ -6744,21 +6744,21 @@
     </row>
     <row r="536" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A536" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B536" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C536">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="537" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A537" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B537" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C537">
         <v>0</v>
@@ -6766,10 +6766,10 @@
     </row>
     <row r="538" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A538" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B538" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C538">
         <v>0</v>
@@ -6777,35 +6777,35 @@
     </row>
     <row r="539" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A539" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B539" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C539">
-        <v>110</v>
+        <v>0</v>
       </c>
     </row>
     <row r="540" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A540" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B540" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C540">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="541" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A541" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B541" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C541">
-        <v>110</v>
+        <v>0</v>
       </c>
     </row>
     <row r="542" spans="1:3" x14ac:dyDescent="0.25">
@@ -6813,26 +6813,26 @@
         <v>149</v>
       </c>
       <c r="B542" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C542">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="543" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A543" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B543" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C543">
-        <v>150</v>
+        <v>60</v>
       </c>
     </row>
     <row r="544" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A544" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B544" s="1" t="s">
         <v>1</v>
@@ -6842,33 +6842,33 @@
       </c>
     </row>
     <row r="545" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A545">
-        <v>721014</v>
+      <c r="A545" t="s">
+        <v>149</v>
       </c>
       <c r="B545" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C545">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="546" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A546">
-        <v>721008</v>
+      <c r="A546" t="s">
+        <v>151</v>
       </c>
       <c r="B546" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C546">
-        <v>60</v>
+        <v>150</v>
       </c>
     </row>
     <row r="547" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A547">
-        <v>721005</v>
+      <c r="A547" t="s">
+        <v>151</v>
       </c>
       <c r="B547" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C547">
         <v>110</v>
@@ -6876,13 +6876,13 @@
     </row>
     <row r="548" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A548">
-        <v>721005</v>
+        <v>721014</v>
       </c>
       <c r="B548" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C548">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="549" spans="1:3" x14ac:dyDescent="0.25">
@@ -6890,7 +6890,7 @@
         <v>721008</v>
       </c>
       <c r="B549" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C549">
         <v>60</v>
@@ -6898,29 +6898,29 @@
     </row>
     <row r="550" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A550">
-        <v>721014</v>
+        <v>721005</v>
       </c>
       <c r="B550" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C550">
-        <v>50</v>
+        <v>110</v>
       </c>
     </row>
     <row r="551" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A551" t="s">
-        <v>152</v>
+      <c r="A551">
+        <v>721005</v>
       </c>
       <c r="B551" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C551">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="552" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A552" t="s">
-        <v>152</v>
+      <c r="A552">
+        <v>721008</v>
       </c>
       <c r="B552" s="1" t="s">
         <v>1</v>
@@ -6931,79 +6931,79 @@
     </row>
     <row r="553" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A553">
-        <v>241040</v>
+        <v>721014</v>
       </c>
       <c r="B553" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C553">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="554" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A554">
-        <v>241020</v>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="554" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A554" t="s">
+        <v>152</v>
       </c>
       <c r="B554" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C554">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="555" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A555">
-        <v>241020</v>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="555" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A555" t="s">
+        <v>152</v>
       </c>
       <c r="B555" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C555">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="556" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="556" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A556">
         <v>241040</v>
       </c>
       <c r="B556" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C556">
-        <v>60</v>
+        <v>120</v>
       </c>
     </row>
     <row r="557" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A557">
-        <v>601138</v>
+        <v>241020</v>
       </c>
       <c r="B557" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C557">
-        <v>110</v>
+        <v>70</v>
       </c>
     </row>
     <row r="558" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A558">
-        <v>601128</v>
+        <v>241020</v>
       </c>
       <c r="B558" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C558">
-        <v>80</v>
+        <v>110</v>
       </c>
     </row>
     <row r="559" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A559">
-        <v>601128</v>
+        <v>241040</v>
       </c>
       <c r="B559" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C559">
-        <v>100</v>
+        <v>60</v>
       </c>
     </row>
     <row r="560" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7011,54 +7011,54 @@
         <v>601138</v>
       </c>
       <c r="B560" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C560">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="561" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A561">
+        <v>601128</v>
+      </c>
+      <c r="B561" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C561">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="562" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A562">
+        <v>601128</v>
+      </c>
+      <c r="B562" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C562">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A563">
+        <v>601138</v>
+      </c>
+      <c r="B563" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C563">
         <v>60</v>
-      </c>
-    </row>
-    <row r="561" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A561" t="s">
-        <v>153</v>
-      </c>
-      <c r="B561" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C561">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="562" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A562" t="s">
-        <v>154</v>
-      </c>
-      <c r="B562" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C562">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A563" t="s">
-        <v>155</v>
-      </c>
-      <c r="B563" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C563">
-        <v>0</v>
       </c>
     </row>
     <row r="564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A564" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B564" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C564">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="565" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7066,20 +7066,53 @@
         <v>154</v>
       </c>
       <c r="B565" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C565">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="566" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A566" t="s">
+        <v>155</v>
+      </c>
+      <c r="B566" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C566">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="567" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A567" t="s">
+        <v>155</v>
+      </c>
+      <c r="B567" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C567">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="568" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A568" t="s">
+        <v>154</v>
+      </c>
+      <c r="B568" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C568">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="569" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A569" t="s">
         <v>153</v>
       </c>
-      <c r="B566" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C566">
+      <c r="B569" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C569">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add: Missing geometrie and correction side
</commit_message>
<xml_diff>
--- a/project/config/profile_config_file.xlsx
+++ b/project/config/profile_config_file.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsochacki\Desktop\Python\Tkinter\production-counting\project\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE59DF8-0FB9-4EF2-B1EA-445367DE920A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{296A6783-A4A2-4B05-A2EC-7A64EF62713B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-195" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="profile_config" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="863" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="865" uniqueCount="177">
   <si>
     <t>GP8280</t>
   </si>
@@ -564,6 +564,9 @@
   </si>
   <si>
     <t>GO2090</t>
+  </si>
+  <si>
+    <t>P29537</t>
   </si>
 </sst>
 </file>
@@ -848,7 +851,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C569"/>
+  <dimension ref="A1:C570"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" customWidth="1"/>
@@ -3458,7 +3461,7 @@
         <v>550801</v>
       </c>
       <c r="B237" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C237">
         <v>90</v>
@@ -3469,7 +3472,7 @@
         <v>553424</v>
       </c>
       <c r="B238" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C238">
         <v>100</v>
@@ -3510,7 +3513,7 @@
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>69</v>
+        <v>176</v>
       </c>
       <c r="B242" s="1" t="s">
         <v>30</v>
@@ -3521,40 +3524,40 @@
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B243" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C243">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B244" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C244">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
+        <v>71</v>
+      </c>
+      <c r="B245" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C245">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A246" t="s">
         <v>72</v>
-      </c>
-      <c r="B245" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C245">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A246">
-        <v>721015</v>
       </c>
       <c r="B246" s="1" t="s">
         <v>30</v>
@@ -3565,7 +3568,7 @@
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247">
-        <v>721009</v>
+        <v>721015</v>
       </c>
       <c r="B247" s="1" t="s">
         <v>30</v>
@@ -3576,7 +3579,7 @@
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248">
-        <v>341040</v>
+        <v>721009</v>
       </c>
       <c r="B248" s="1" t="s">
         <v>30</v>
@@ -3587,7 +3590,7 @@
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249">
-        <v>341030</v>
+        <v>341040</v>
       </c>
       <c r="B249" s="1" t="s">
         <v>30</v>
@@ -3601,15 +3604,15 @@
         <v>341030</v>
       </c>
       <c r="B250" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C250">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251">
-        <v>341040</v>
+        <v>341030</v>
       </c>
       <c r="B251" s="1" t="s">
         <v>1</v>
@@ -3620,7 +3623,7 @@
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252">
-        <v>721009</v>
+        <v>341040</v>
       </c>
       <c r="B252" s="1" t="s">
         <v>1</v>
@@ -3631,7 +3634,7 @@
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253">
-        <v>721015</v>
+        <v>721009</v>
       </c>
       <c r="B253" s="1" t="s">
         <v>1</v>
@@ -3641,8 +3644,8 @@
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A254" t="s">
-        <v>72</v>
+      <c r="A254">
+        <v>721015</v>
       </c>
       <c r="B254" s="1" t="s">
         <v>1</v>
@@ -3653,7 +3656,7 @@
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B255" s="1" t="s">
         <v>1</v>
@@ -3664,46 +3667,46 @@
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B256" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C256">
-        <v>110</v>
+        <v>55</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B257" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C257">
-        <v>0</v>
+        <v>110</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B258" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C258">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B259" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C259">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
@@ -3711,37 +3714,37 @@
         <v>74</v>
       </c>
       <c r="B260" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C260">
-        <v>75</v>
+        <v>0</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B261" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C261">
-        <v>90</v>
+        <v>75</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B262" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C262">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="263" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B263" s="1" t="s">
         <v>30</v>
@@ -3752,7 +3755,7 @@
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B264" s="1" t="s">
         <v>30</v>
@@ -3762,58 +3765,58 @@
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A265">
-        <v>720024</v>
+      <c r="A265" t="s">
+        <v>77</v>
       </c>
       <c r="B265" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C265">
-        <v>90</v>
+        <v>70</v>
       </c>
     </row>
     <row r="266" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A266">
+        <v>720024</v>
+      </c>
+      <c r="B266" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C266">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A267">
         <v>720022</v>
       </c>
-      <c r="B266" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C266">
+      <c r="B267" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C267">
         <v>70</v>
-      </c>
-    </row>
-    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A267" t="s">
-        <v>78</v>
-      </c>
-      <c r="B267" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C267">
-        <v>80</v>
       </c>
     </row>
     <row r="268" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
+        <v>78</v>
+      </c>
+      <c r="B268" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C268">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="269" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A269" t="s">
         <v>79</v>
       </c>
-      <c r="B268" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C268">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="269" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A269">
-        <v>661000</v>
-      </c>
       <c r="B269" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C269">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.25">
@@ -3821,15 +3824,15 @@
         <v>661000</v>
       </c>
       <c r="B270" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C270">
         <v>70</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A271" t="s">
-        <v>78</v>
+      <c r="A271">
+        <v>661000</v>
       </c>
       <c r="B271" s="1" t="s">
         <v>1</v>
@@ -3840,7 +3843,7 @@
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B272" s="1" t="s">
         <v>1</v>
@@ -3850,8 +3853,8 @@
       </c>
     </row>
     <row r="273" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A273">
-        <v>720022</v>
+      <c r="A273" t="s">
+        <v>79</v>
       </c>
       <c r="B273" s="1" t="s">
         <v>1</v>
@@ -3862,7 +3865,7 @@
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A274">
-        <v>720024</v>
+        <v>720022</v>
       </c>
       <c r="B274" s="1" t="s">
         <v>1</v>
@@ -3872,8 +3875,8 @@
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A275" t="s">
-        <v>77</v>
+      <c r="A275">
+        <v>720024</v>
       </c>
       <c r="B275" s="1" t="s">
         <v>1</v>
@@ -3884,46 +3887,46 @@
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B276" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C276">
-        <v>110</v>
+        <v>70</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B277" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C277">
-        <v>0</v>
+        <v>110</v>
       </c>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
+        <v>75</v>
+      </c>
+      <c r="B278" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C278">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="279" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A279" t="s">
         <v>80</v>
       </c>
-      <c r="B278" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C278">
+      <c r="B279" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C279">
         <v>100</v>
-      </c>
-    </row>
-    <row r="279" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A279">
-        <v>416210</v>
-      </c>
-      <c r="B279" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C279">
-        <v>0</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.25">
@@ -3931,54 +3934,54 @@
         <v>416210</v>
       </c>
       <c r="B280" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C280">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A281">
+        <v>416210</v>
+      </c>
+      <c r="B281" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C281">
         <v>100</v>
       </c>
     </row>
-    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A281" t="s">
+    <row r="282" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A282" t="s">
         <v>80</v>
       </c>
-      <c r="B281" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C281">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="282" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A282">
-        <v>406210</v>
-      </c>
       <c r="B282" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C282">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283">
-        <v>650050</v>
+        <v>406210</v>
       </c>
       <c r="B283" s="1" t="s">
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="C283">
-        <v>120</v>
+        <v>100</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A284">
-        <v>650040</v>
+        <v>650050</v>
       </c>
       <c r="B284" s="1" t="s">
         <v>81</v>
       </c>
       <c r="C284">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
@@ -3986,10 +3989,10 @@
         <v>650040</v>
       </c>
       <c r="B285" s="1" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="C285">
-        <v>140</v>
+        <v>90</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.25">
@@ -3997,21 +4000,21 @@
         <v>650040</v>
       </c>
       <c r="B286" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C286">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A287">
-        <v>650050</v>
+        <v>650040</v>
       </c>
       <c r="B287" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C287">
-        <v>140</v>
+        <v>150</v>
       </c>
     </row>
     <row r="288" spans="1:3" x14ac:dyDescent="0.25">
@@ -4019,21 +4022,21 @@
         <v>650050</v>
       </c>
       <c r="B288" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C288">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A289">
-        <v>650020</v>
+        <v>650050</v>
       </c>
       <c r="B289" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C289">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.25">
@@ -4041,21 +4044,21 @@
         <v>650020</v>
       </c>
       <c r="B290" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C290">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="291" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A291">
-        <v>600138</v>
+        <v>650020</v>
       </c>
       <c r="B291" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C291">
-        <v>170</v>
+        <v>100</v>
       </c>
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.25">
@@ -4063,26 +4066,26 @@
         <v>600138</v>
       </c>
       <c r="B292" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C292">
-        <v>150</v>
+        <v>170</v>
       </c>
     </row>
     <row r="293" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A293">
-        <v>600121</v>
+        <v>600138</v>
       </c>
       <c r="B293" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C293">
-        <v>140</v>
+        <v>150</v>
       </c>
     </row>
     <row r="294" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A294">
-        <v>600127</v>
+        <v>600121</v>
       </c>
       <c r="B294" s="1" t="s">
         <v>30</v>
@@ -4093,7 +4096,7 @@
     </row>
     <row r="295" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A295">
-        <v>600227</v>
+        <v>600127</v>
       </c>
       <c r="B295" s="1" t="s">
         <v>30</v>
@@ -4107,26 +4110,26 @@
         <v>600227</v>
       </c>
       <c r="B296" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C296">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
     <row r="297" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A297">
-        <v>600127</v>
+        <v>600227</v>
       </c>
       <c r="B297" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C297">
-        <v>90</v>
+        <v>150</v>
       </c>
     </row>
     <row r="298" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A298">
-        <v>600121</v>
+        <v>600127</v>
       </c>
       <c r="B298" s="1" t="s">
         <v>1</v>
@@ -4137,13 +4140,13 @@
     </row>
     <row r="299" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A299">
-        <v>600128</v>
+        <v>600121</v>
       </c>
       <c r="B299" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C299">
-        <v>150</v>
+        <v>90</v>
       </c>
     </row>
     <row r="300" spans="1:3" x14ac:dyDescent="0.25">
@@ -4151,21 +4154,21 @@
         <v>600128</v>
       </c>
       <c r="B300" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C300">
-        <v>70</v>
+        <v>150</v>
       </c>
     </row>
     <row r="301" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A301">
-        <v>650030</v>
+        <v>600128</v>
       </c>
       <c r="B301" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C301">
-        <v>170</v>
+        <v>70</v>
       </c>
     </row>
     <row r="302" spans="1:3" x14ac:dyDescent="0.25">
@@ -4173,21 +4176,21 @@
         <v>650030</v>
       </c>
       <c r="B302" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C302">
-        <v>70</v>
+        <v>170</v>
       </c>
     </row>
     <row r="303" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A303">
-        <v>660000</v>
+        <v>650030</v>
       </c>
       <c r="B303" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C303">
-        <v>120</v>
+        <v>70</v>
       </c>
     </row>
     <row r="304" spans="1:3" x14ac:dyDescent="0.25">
@@ -4195,21 +4198,21 @@
         <v>660000</v>
       </c>
       <c r="B304" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C304">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A305">
+        <v>660000</v>
+      </c>
+      <c r="B305" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C305">
         <v>80</v>
-      </c>
-    </row>
-    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A305" t="s">
-        <v>82</v>
-      </c>
-      <c r="B305" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C305">
-        <v>110</v>
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.25">
@@ -4217,18 +4220,18 @@
         <v>82</v>
       </c>
       <c r="B306" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C306">
-        <v>0</v>
+        <v>110</v>
       </c>
     </row>
     <row r="307" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B307" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C307">
         <v>0</v>
@@ -4239,7 +4242,7 @@
         <v>83</v>
       </c>
       <c r="B308" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C308">
         <v>0</v>
@@ -4250,32 +4253,32 @@
         <v>83</v>
       </c>
       <c r="B309" s="1" t="s">
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="C309">
-        <v>120</v>
+        <v>0</v>
       </c>
     </row>
     <row r="310" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B310" s="1" t="s">
         <v>81</v>
       </c>
       <c r="C310">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="311" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A311">
-        <v>406670</v>
+      <c r="A311" t="s">
+        <v>82</v>
       </c>
       <c r="B311" s="1" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="C311">
-        <v>110</v>
+        <v>0</v>
       </c>
     </row>
     <row r="312" spans="1:3" x14ac:dyDescent="0.25">
@@ -4283,32 +4286,32 @@
         <v>406670</v>
       </c>
       <c r="B312" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C312">
-        <v>0</v>
+        <v>110</v>
       </c>
     </row>
     <row r="313" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A313">
+        <v>406670</v>
+      </c>
+      <c r="B313" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C313">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A314">
         <v>406316</v>
       </c>
-      <c r="B313" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C313">
+      <c r="B314" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C314">
         <v>120</v>
-      </c>
-    </row>
-    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A314" t="s">
-        <v>84</v>
-      </c>
-      <c r="B314" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C314">
-        <v>80</v>
       </c>
     </row>
     <row r="315" spans="1:3" x14ac:dyDescent="0.25">
@@ -4316,21 +4319,21 @@
         <v>84</v>
       </c>
       <c r="B315" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C315">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="316" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B316" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C316">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="317" spans="1:3" x14ac:dyDescent="0.25">
@@ -4338,59 +4341,59 @@
         <v>85</v>
       </c>
       <c r="B317" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C317">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="318" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
+        <v>85</v>
+      </c>
+      <c r="B318" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C318">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="319" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A319" t="s">
         <v>86</v>
       </c>
-      <c r="B318" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C318">
+      <c r="B319" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C319">
         <v>60</v>
       </c>
     </row>
-    <row r="319" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A319">
+    <row r="320" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A320">
         <v>550800</v>
       </c>
-      <c r="B319" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C319">
+      <c r="B320" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C320">
         <v>80</v>
-      </c>
-    </row>
-    <row r="320" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A320" t="s">
-        <v>87</v>
-      </c>
-      <c r="B320" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C320">
-        <v>90</v>
       </c>
     </row>
     <row r="321" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B321" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C321">
-        <v>60</v>
+        <v>90</v>
       </c>
     </row>
     <row r="322" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B322" s="1" t="s">
         <v>30</v>
@@ -4401,18 +4404,18 @@
     </row>
     <row r="323" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B323" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C323">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="324" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B324" s="1" t="s">
         <v>30</v>
@@ -4423,73 +4426,73 @@
     </row>
     <row r="325" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B325" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C325">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="326" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
+        <v>92</v>
+      </c>
+      <c r="B326" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C326">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="327" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A327" t="s">
         <v>93</v>
       </c>
-      <c r="B326" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C326">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="327" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A327">
+      <c r="B327" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C327">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="328" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A328">
         <v>720023</v>
       </c>
-      <c r="B327" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C327">
+      <c r="B328" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C328">
         <v>80</v>
       </c>
     </row>
-    <row r="328" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A328" t="s">
+    <row r="329" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A329" t="s">
         <v>94</v>
       </c>
-      <c r="B328" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C328">
+      <c r="B329" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C329">
         <v>70</v>
-      </c>
-    </row>
-    <row r="329" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A329">
-        <v>240040</v>
-      </c>
-      <c r="B329" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C329">
-        <v>60</v>
       </c>
     </row>
     <row r="330" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A330">
-        <v>240030</v>
+        <v>240040</v>
       </c>
       <c r="B330" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C330">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="331" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A331">
-        <v>240020</v>
+        <v>240030</v>
       </c>
       <c r="B331" s="1" t="s">
         <v>30</v>
@@ -4503,26 +4506,26 @@
         <v>240020</v>
       </c>
       <c r="B332" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C332">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="333" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A333">
-        <v>240030</v>
+        <v>240020</v>
       </c>
       <c r="B333" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C333">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="334" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A334">
-        <v>240040</v>
+        <v>240030</v>
       </c>
       <c r="B334" s="1" t="s">
         <v>1</v>
@@ -4532,8 +4535,8 @@
       </c>
     </row>
     <row r="335" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A335" t="s">
-        <v>94</v>
+      <c r="A335">
+        <v>240040</v>
       </c>
       <c r="B335" s="1" t="s">
         <v>1</v>
@@ -4543,19 +4546,19 @@
       </c>
     </row>
     <row r="336" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A336">
+      <c r="A336" t="s">
+        <v>94</v>
+      </c>
+      <c r="B336" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C336">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="337" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A337">
         <v>720023</v>
-      </c>
-      <c r="B336" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C336">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="337" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A337" t="s">
-        <v>93</v>
       </c>
       <c r="B337" s="1" t="s">
         <v>1</v>
@@ -4566,40 +4569,40 @@
     </row>
     <row r="338" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B338" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C338">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="339" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B339" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C339">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="340" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B340" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C340">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="341" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B341" s="1" t="s">
         <v>1</v>
@@ -4610,18 +4613,18 @@
     </row>
     <row r="342" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B342" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C342">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
     <row r="343" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B343" s="1" t="s">
         <v>1</v>
@@ -4632,35 +4635,35 @@
     </row>
     <row r="344" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="B344" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C344">
-        <v>80</v>
+        <v>50</v>
       </c>
     </row>
     <row r="345" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B345" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C345">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="346" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B346" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C346">
-        <v>45</v>
+        <v>0</v>
       </c>
     </row>
     <row r="347" spans="1:3" x14ac:dyDescent="0.25">
@@ -4668,15 +4671,15 @@
         <v>97</v>
       </c>
       <c r="B347" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C347">
-        <v>60</v>
+        <v>45</v>
       </c>
     </row>
     <row r="348" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B348" s="1" t="s">
         <v>1</v>
@@ -4687,40 +4690,40 @@
     </row>
     <row r="349" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
+        <v>96</v>
+      </c>
+      <c r="B349" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C349">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="350" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A350" t="s">
         <v>95</v>
       </c>
-      <c r="B349" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C349">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="350" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A350">
-        <v>722010</v>
-      </c>
       <c r="B350" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C350">
-        <v>80</v>
+        <v>30</v>
       </c>
     </row>
     <row r="351" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A351">
-        <v>722005</v>
+        <v>722010</v>
       </c>
       <c r="B351" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C351">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="352" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A352">
-        <v>722006</v>
+        <v>722005</v>
       </c>
       <c r="B352" s="1" t="s">
         <v>30</v>
@@ -4731,13 +4734,13 @@
     </row>
     <row r="353" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A353">
-        <v>722000</v>
+        <v>722006</v>
       </c>
       <c r="B353" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C353">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="354" spans="1:3" x14ac:dyDescent="0.25">
@@ -4745,7 +4748,7 @@
         <v>722000</v>
       </c>
       <c r="B354" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C354">
         <v>60</v>
@@ -4753,18 +4756,18 @@
     </row>
     <row r="355" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A355">
-        <v>722006</v>
+        <v>722000</v>
       </c>
       <c r="B355" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C355">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="356" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A356">
-        <v>722005</v>
+        <v>722006</v>
       </c>
       <c r="B356" s="1" t="s">
         <v>1</v>
@@ -4775,40 +4778,40 @@
     </row>
     <row r="357" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A357">
+        <v>722005</v>
+      </c>
+      <c r="B357" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C357">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="358" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A358">
         <v>722010</v>
       </c>
-      <c r="B357" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C357">
+      <c r="B358" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C358">
         <v>50</v>
-      </c>
-    </row>
-    <row r="358" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A358" t="s">
-        <v>98</v>
-      </c>
-      <c r="B358" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C358">
-        <v>80</v>
       </c>
     </row>
     <row r="359" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B359" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C359">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="360" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B360" s="1" t="s">
         <v>30</v>
@@ -4819,13 +4822,13 @@
     </row>
     <row r="361" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B361" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C361">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="362" spans="1:3" x14ac:dyDescent="0.25">
@@ -4833,7 +4836,7 @@
         <v>101</v>
       </c>
       <c r="B362" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C362">
         <v>60</v>
@@ -4841,29 +4844,29 @@
     </row>
     <row r="363" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B363" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C363">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="364" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B364" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C364">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="365" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B365" s="1" t="s">
         <v>1</v>
@@ -4874,40 +4877,40 @@
     </row>
     <row r="366" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="B366" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C366">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="367" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B367" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C367">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="368" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B368" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C368">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="369" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B369" s="1" t="s">
         <v>30</v>
@@ -4921,26 +4924,26 @@
         <v>105</v>
       </c>
       <c r="B370" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C370">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="371" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B371" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C371">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="372" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B372" s="1" t="s">
         <v>1</v>
@@ -4951,35 +4954,35 @@
     </row>
     <row r="373" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B373" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C373">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="374" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B374" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C374">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="375" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B375" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C375">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="376" spans="1:3" x14ac:dyDescent="0.25">
@@ -4987,70 +4990,70 @@
         <v>107</v>
       </c>
       <c r="B376" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C376">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="377" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
+        <v>107</v>
+      </c>
+      <c r="B377" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C377">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="378" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A378" t="s">
         <v>106</v>
       </c>
-      <c r="B377" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C377">
+      <c r="B378" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C378">
         <v>60</v>
-      </c>
-    </row>
-    <row r="378" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A378">
-        <v>406010</v>
-      </c>
-      <c r="B378" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C378">
-        <v>120</v>
       </c>
     </row>
     <row r="379" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A379">
-        <v>406321</v>
+        <v>406010</v>
       </c>
       <c r="B379" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C379">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="380" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A380">
-        <v>406660</v>
+        <v>406321</v>
       </c>
       <c r="B380" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C380">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="381" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A381">
-        <v>406329</v>
+        <v>406660</v>
       </c>
       <c r="B381" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C381">
-        <v>150</v>
+        <v>120</v>
       </c>
     </row>
     <row r="382" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A382">
-        <v>406325</v>
+        <v>406329</v>
       </c>
       <c r="B382" s="1" t="s">
         <v>1</v>
@@ -5061,13 +5064,13 @@
     </row>
     <row r="383" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A383">
-        <v>416240</v>
+        <v>406325</v>
       </c>
       <c r="B383" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C383">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="384" spans="1:3" x14ac:dyDescent="0.25">
@@ -5075,15 +5078,15 @@
         <v>416240</v>
       </c>
       <c r="B384" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C384">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="385" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A385" t="s">
-        <v>108</v>
+      <c r="A385">
+        <v>416240</v>
       </c>
       <c r="B385" s="1" t="s">
         <v>1</v>
@@ -5094,10 +5097,10 @@
     </row>
     <row r="386" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B386" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C386">
         <v>100</v>
@@ -5108,21 +5111,21 @@
         <v>109</v>
       </c>
       <c r="B387" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C387">
-        <v>120</v>
+        <v>100</v>
       </c>
     </row>
     <row r="388" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B388" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C388">
-        <v>100</v>
+        <v>120</v>
       </c>
     </row>
     <row r="389" spans="1:3" x14ac:dyDescent="0.25">
@@ -5130,7 +5133,7 @@
         <v>110</v>
       </c>
       <c r="B389" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C389">
         <v>100</v>
@@ -5138,10 +5141,10 @@
     </row>
     <row r="390" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B390" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C390">
         <v>100</v>
@@ -5152,18 +5155,18 @@
         <v>111</v>
       </c>
       <c r="B391" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C391">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="392" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B392" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C392">
         <v>90</v>
@@ -5174,21 +5177,21 @@
         <v>112</v>
       </c>
       <c r="B393" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C393">
-        <v>130</v>
+        <v>90</v>
       </c>
     </row>
     <row r="394" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B394" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C394">
-        <v>100</v>
+        <v>130</v>
       </c>
     </row>
     <row r="395" spans="1:3" x14ac:dyDescent="0.25">
@@ -5196,21 +5199,21 @@
         <v>113</v>
       </c>
       <c r="B395" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C395">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="396" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A396" t="s">
+        <v>113</v>
+      </c>
+      <c r="B396" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C396">
         <v>130</v>
-      </c>
-    </row>
-    <row r="396" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A396">
-        <v>242320</v>
-      </c>
-      <c r="B396" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C396">
-        <v>100</v>
       </c>
     </row>
     <row r="397" spans="1:3" x14ac:dyDescent="0.25">
@@ -5218,7 +5221,7 @@
         <v>242320</v>
       </c>
       <c r="B397" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C397">
         <v>100</v>
@@ -5226,13 +5229,13 @@
     </row>
     <row r="398" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A398">
-        <v>651050</v>
+        <v>242320</v>
       </c>
       <c r="B398" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C398">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="399" spans="1:3" x14ac:dyDescent="0.25">
@@ -5240,7 +5243,7 @@
         <v>651050</v>
       </c>
       <c r="B399" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C399">
         <v>110</v>
@@ -5248,13 +5251,13 @@
     </row>
     <row r="400" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A400">
-        <v>730010</v>
+        <v>651050</v>
       </c>
       <c r="B400" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C400">
-        <v>100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="401" spans="1:3" x14ac:dyDescent="0.25">
@@ -5262,7 +5265,7 @@
         <v>730010</v>
       </c>
       <c r="B401" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C401">
         <v>100</v>
@@ -5270,10 +5273,10 @@
     </row>
     <row r="402" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A402">
-        <v>731020</v>
+        <v>730010</v>
       </c>
       <c r="B402" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C402">
         <v>100</v>
@@ -5284,21 +5287,21 @@
         <v>731020</v>
       </c>
       <c r="B403" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C403">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="404" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A404">
-        <v>476273</v>
+        <v>731020</v>
       </c>
       <c r="B404" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C404">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="405" spans="1:3" x14ac:dyDescent="0.25">
@@ -5306,21 +5309,21 @@
         <v>476273</v>
       </c>
       <c r="B405" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C405">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="406" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A406" t="s">
-        <v>114</v>
+      <c r="A406">
+        <v>476273</v>
       </c>
       <c r="B406" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C406">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="407" spans="1:3" x14ac:dyDescent="0.25">
@@ -5328,21 +5331,21 @@
         <v>114</v>
       </c>
       <c r="B407" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C407">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="408" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A408">
-        <v>466009</v>
+      <c r="A408" t="s">
+        <v>114</v>
       </c>
       <c r="B408" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C408">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="409" spans="1:3" x14ac:dyDescent="0.25">
@@ -5350,21 +5353,21 @@
         <v>466009</v>
       </c>
       <c r="B409" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C409">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="410" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A410">
-        <v>416273</v>
+        <v>466009</v>
       </c>
       <c r="B410" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C410">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="411" spans="1:3" x14ac:dyDescent="0.25">
@@ -5372,21 +5375,21 @@
         <v>416273</v>
       </c>
       <c r="B411" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C411">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="412" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A412">
-        <v>466023</v>
+        <v>416273</v>
       </c>
       <c r="B412" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C412">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="413" spans="1:3" x14ac:dyDescent="0.25">
@@ -5394,21 +5397,21 @@
         <v>466023</v>
       </c>
       <c r="B413" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C413">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="414" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A414">
-        <v>426200</v>
+        <v>466023</v>
       </c>
       <c r="B414" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C414">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="415" spans="1:3" x14ac:dyDescent="0.25">
@@ -5416,21 +5419,21 @@
         <v>426200</v>
       </c>
       <c r="B415" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C415">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="416" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A416">
-        <v>406272</v>
+        <v>426200</v>
       </c>
       <c r="B416" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C416">
-        <v>60</v>
+        <v>0</v>
       </c>
     </row>
     <row r="417" spans="1:3" x14ac:dyDescent="0.25">
@@ -5438,21 +5441,21 @@
         <v>406272</v>
       </c>
       <c r="B417" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C417">
-        <v>0</v>
+        <v>60</v>
       </c>
     </row>
     <row r="418" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A418" t="s">
-        <v>115</v>
+      <c r="A418">
+        <v>406272</v>
       </c>
       <c r="B418" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C418">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="419" spans="1:3" x14ac:dyDescent="0.25">
@@ -5460,18 +5463,18 @@
         <v>115</v>
       </c>
       <c r="B419" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C419">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="420" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B420" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C420">
         <v>80</v>
@@ -5482,7 +5485,7 @@
         <v>116</v>
       </c>
       <c r="B421" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C421">
         <v>80</v>
@@ -5490,10 +5493,10 @@
     </row>
     <row r="422" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B422" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C422">
         <v>80</v>
@@ -5504,147 +5507,147 @@
         <v>117</v>
       </c>
       <c r="B423" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C423">
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="424" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A424">
-        <v>416338</v>
+      <c r="A424" t="s">
+        <v>117</v>
       </c>
       <c r="B424" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C424">
-        <v>150</v>
+        <v>0</v>
       </c>
     </row>
     <row r="425" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A425">
-        <v>416331</v>
+        <v>416338</v>
       </c>
       <c r="B425" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C425">
-        <v>200</v>
+        <v>150</v>
       </c>
     </row>
     <row r="426" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A426">
-        <v>416065</v>
+        <v>416331</v>
       </c>
       <c r="B426" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C426">
-        <v>90</v>
+        <v>200</v>
       </c>
     </row>
     <row r="427" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A427">
-        <v>416067</v>
+        <v>416065</v>
       </c>
       <c r="B427" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C427">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="428" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A428">
-        <v>416086</v>
+        <v>416067</v>
       </c>
       <c r="B428" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C428">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="429" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A429">
+        <v>416086</v>
+      </c>
+      <c r="B429" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C429">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="430" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A430">
         <v>416096</v>
       </c>
-      <c r="B429" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C429">
+      <c r="B430" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C430">
         <v>120</v>
       </c>
     </row>
-    <row r="430" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A430" t="s">
+    <row r="431" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A431" t="s">
         <v>118</v>
       </c>
-      <c r="B430" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C430">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="431" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A431">
-        <v>666003</v>
-      </c>
       <c r="B431" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C431">
-        <v>120</v>
+        <v>90</v>
       </c>
     </row>
     <row r="432" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A432">
+        <v>666003</v>
+      </c>
+      <c r="B432" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C432">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="433" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A433">
         <v>666002</v>
       </c>
-      <c r="B432" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C432">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="433" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A433" t="s">
+      <c r="B433" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C433">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="434" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A434" t="s">
         <v>119</v>
       </c>
-      <c r="B433" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C433">
+      <c r="B434" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C434">
         <v>85</v>
-      </c>
-    </row>
-    <row r="434" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A434">
-        <v>416070</v>
-      </c>
-      <c r="B434" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C434">
-        <v>90</v>
       </c>
     </row>
     <row r="435" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A435">
+        <v>416070</v>
+      </c>
+      <c r="B435" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C435">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="436" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A436">
         <v>416069</v>
-      </c>
-      <c r="B435" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C435">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="436" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A436" t="s">
-        <v>120</v>
       </c>
       <c r="B436" s="1" t="s">
         <v>1</v>
@@ -5654,8 +5657,8 @@
       </c>
     </row>
     <row r="437" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A437">
-        <v>406340</v>
+      <c r="A437" t="s">
+        <v>120</v>
       </c>
       <c r="B437" s="1" t="s">
         <v>1</v>
@@ -5666,7 +5669,7 @@
     </row>
     <row r="438" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A438">
-        <v>416301</v>
+        <v>406340</v>
       </c>
       <c r="B438" s="1" t="s">
         <v>1</v>
@@ -5677,35 +5680,35 @@
     </row>
     <row r="439" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A439">
-        <v>416119</v>
+        <v>416301</v>
       </c>
       <c r="B439" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C439">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="440" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A440">
-        <v>406081</v>
+        <v>416119</v>
       </c>
       <c r="B440" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C440">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="441" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A441">
-        <v>416068</v>
+        <v>406081</v>
       </c>
       <c r="B441" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C441">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="442" spans="1:3" x14ac:dyDescent="0.25">
@@ -5713,48 +5716,48 @@
         <v>416068</v>
       </c>
       <c r="B442" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C442">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="443" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A443">
-        <v>736315</v>
+        <v>416068</v>
       </c>
       <c r="B443" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C443">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="444" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A444">
+        <v>736315</v>
+      </c>
+      <c r="B444" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C444">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="445" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A445">
         <v>736334</v>
       </c>
-      <c r="B444" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C444">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="445" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A445" t="s">
+      <c r="B445" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C445">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="446" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A446" t="s">
         <v>121</v>
-      </c>
-      <c r="B445" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C445">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="446" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A446">
-        <v>406307</v>
       </c>
       <c r="B446" s="1" t="s">
         <v>1</v>
@@ -5765,7 +5768,7 @@
     </row>
     <row r="447" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A447">
-        <v>466400</v>
+        <v>406307</v>
       </c>
       <c r="B447" s="1" t="s">
         <v>1</v>
@@ -5776,13 +5779,13 @@
     </row>
     <row r="448" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A448">
-        <v>416139</v>
+        <v>466400</v>
       </c>
       <c r="B448" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C448">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="449" spans="1:3" x14ac:dyDescent="0.25">
@@ -5790,7 +5793,7 @@
         <v>416139</v>
       </c>
       <c r="B449" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C449">
         <v>80</v>
@@ -5798,7 +5801,7 @@
     </row>
     <row r="450" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A450">
-        <v>416148</v>
+        <v>416139</v>
       </c>
       <c r="B450" s="1" t="s">
         <v>1</v>
@@ -5808,30 +5811,30 @@
       </c>
     </row>
     <row r="451" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A451" t="s">
-        <v>122</v>
+      <c r="A451">
+        <v>416148</v>
       </c>
       <c r="B451" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C451">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="452" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B452" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C452">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="453" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A453" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B453" s="1" t="s">
         <v>1</v>
@@ -5842,7 +5845,7 @@
     </row>
     <row r="454" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B454" s="1" t="s">
         <v>1</v>
@@ -5853,40 +5856,40 @@
     </row>
     <row r="455" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B455" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C455">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="456" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B456" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C456">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="457" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B457" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C457">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="458" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
-        <v>171</v>
+        <v>128</v>
       </c>
       <c r="B458" s="1" t="s">
         <v>1</v>
@@ -5896,30 +5899,30 @@
       </c>
     </row>
     <row r="459" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A459">
+      <c r="A459" t="s">
+        <v>171</v>
+      </c>
+      <c r="B459" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C459">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="460" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A460">
         <v>406310</v>
       </c>
-      <c r="B459" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C459">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="460" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A460" t="s">
+      <c r="B460" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C460">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="461" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A461" t="s">
         <v>129</v>
-      </c>
-      <c r="B460" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C460">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="461" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A461">
-        <v>416180</v>
       </c>
       <c r="B461" s="1" t="s">
         <v>1</v>
@@ -5930,7 +5933,7 @@
     </row>
     <row r="462" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A462">
-        <v>606180</v>
+        <v>416180</v>
       </c>
       <c r="B462" s="1" t="s">
         <v>1</v>
@@ -5941,7 +5944,7 @@
     </row>
     <row r="463" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A463">
-        <v>656310</v>
+        <v>606180</v>
       </c>
       <c r="B463" s="1" t="s">
         <v>1</v>
@@ -5952,7 +5955,7 @@
     </row>
     <row r="464" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A464">
-        <v>416311</v>
+        <v>656310</v>
       </c>
       <c r="B464" s="1" t="s">
         <v>1</v>
@@ -5963,7 +5966,7 @@
     </row>
     <row r="465" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A465">
-        <v>406157</v>
+        <v>416311</v>
       </c>
       <c r="B465" s="1" t="s">
         <v>1</v>
@@ -5974,7 +5977,7 @@
     </row>
     <row r="466" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A466">
-        <v>416182</v>
+        <v>406157</v>
       </c>
       <c r="B466" s="1" t="s">
         <v>1</v>
@@ -5985,18 +5988,18 @@
     </row>
     <row r="467" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A467">
-        <v>406315</v>
+        <v>416182</v>
       </c>
       <c r="B467" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C467">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="468" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A468">
-        <v>406312</v>
+        <v>406315</v>
       </c>
       <c r="B468" s="1" t="s">
         <v>1</v>
@@ -6006,19 +6009,19 @@
       </c>
     </row>
     <row r="469" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A469" t="s">
-        <v>130</v>
+      <c r="A469">
+        <v>406312</v>
       </c>
       <c r="B469" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C469">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="470" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B470" s="1" t="s">
         <v>30</v>
@@ -6032,15 +6035,15 @@
         <v>131</v>
       </c>
       <c r="B471" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C471">
-        <v>70</v>
+        <v>90</v>
       </c>
     </row>
     <row r="472" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B472" s="1" t="s">
         <v>1</v>
@@ -6050,14 +6053,14 @@
       </c>
     </row>
     <row r="473" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A473">
-        <v>762013</v>
+      <c r="A473" t="s">
+        <v>130</v>
       </c>
       <c r="B473" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C473">
-        <v>85</v>
+        <v>70</v>
       </c>
     </row>
     <row r="474" spans="1:3" x14ac:dyDescent="0.25">
@@ -6065,21 +6068,21 @@
         <v>762013</v>
       </c>
       <c r="B474" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C474">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="475" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A475">
+        <v>762013</v>
+      </c>
+      <c r="B475" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C475">
         <v>60</v>
-      </c>
-    </row>
-    <row r="475" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A475" t="s">
-        <v>132</v>
-      </c>
-      <c r="B475" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C475">
-        <v>90</v>
       </c>
     </row>
     <row r="476" spans="1:3" x14ac:dyDescent="0.25">
@@ -6087,21 +6090,21 @@
         <v>132</v>
       </c>
       <c r="B476" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C476">
-        <v>60</v>
+        <v>90</v>
       </c>
     </row>
     <row r="477" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B477" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C477">
-        <v>90</v>
+        <v>60</v>
       </c>
     </row>
     <row r="478" spans="1:3" x14ac:dyDescent="0.25">
@@ -6109,21 +6112,21 @@
         <v>133</v>
       </c>
       <c r="B478" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C478">
-        <v>60</v>
+        <v>90</v>
       </c>
     </row>
     <row r="479" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B479" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C479">
-        <v>100</v>
+        <v>60</v>
       </c>
     </row>
     <row r="480" spans="1:3" x14ac:dyDescent="0.25">
@@ -6131,21 +6134,21 @@
         <v>134</v>
       </c>
       <c r="B480" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C480">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="481" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A481" t="s">
+        <v>134</v>
+      </c>
+      <c r="B481" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C481">
         <v>60</v>
-      </c>
-    </row>
-    <row r="481" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A481">
-        <v>242020</v>
-      </c>
-      <c r="B481" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C481">
-        <v>70</v>
       </c>
     </row>
     <row r="482" spans="1:3" x14ac:dyDescent="0.25">
@@ -6153,21 +6156,21 @@
         <v>242020</v>
       </c>
       <c r="B482" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C482">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="483" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A483">
-        <v>602010</v>
+        <v>242020</v>
       </c>
       <c r="B483" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C483">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="484" spans="1:3" x14ac:dyDescent="0.25">
@@ -6175,21 +6178,21 @@
         <v>602010</v>
       </c>
       <c r="B484" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C484">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="485" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A485">
-        <v>652010</v>
+        <v>602010</v>
       </c>
       <c r="B485" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C485">
-        <v>80</v>
+        <v>60</v>
       </c>
     </row>
     <row r="486" spans="1:3" x14ac:dyDescent="0.25">
@@ -6197,37 +6200,37 @@
         <v>652010</v>
       </c>
       <c r="B486" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C486">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="487" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A487">
+        <v>652010</v>
+      </c>
+      <c r="B487" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C487">
         <v>60</v>
-      </c>
-    </row>
-    <row r="487" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A487" t="s">
-        <v>135</v>
-      </c>
-      <c r="B487" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C487">
-        <v>70</v>
       </c>
     </row>
     <row r="488" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B488" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C488">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="489" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A489" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B489" s="1" t="s">
         <v>1</v>
@@ -6238,7 +6241,7 @@
     </row>
     <row r="490" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A490" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B490" s="1" t="s">
         <v>1</v>
@@ -6249,29 +6252,29 @@
     </row>
     <row r="491" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A491" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B491" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C491">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="492" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A492" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B492" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C492">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="493" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A493" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B493" s="1" t="s">
         <v>56</v>
@@ -6282,7 +6285,7 @@
     </row>
     <row r="494" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A494" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B494" s="1" t="s">
         <v>56</v>
@@ -6296,26 +6299,26 @@
         <v>138</v>
       </c>
       <c r="B495" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C495">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="496" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A496" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B496" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C496">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="497" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A497" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B497" s="1" t="s">
         <v>30</v>
@@ -6326,7 +6329,7 @@
     </row>
     <row r="498" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A498" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B498" s="1" t="s">
         <v>30</v>
@@ -6337,29 +6340,29 @@
     </row>
     <row r="499" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A499" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B499" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C499">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="500" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A500" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B500" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C500">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="501" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A501" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B501" s="1" t="s">
         <v>1</v>
@@ -6370,29 +6373,29 @@
     </row>
     <row r="502" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A502" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B502" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C502">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="503" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A503" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B503" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C503">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="504" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A504" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B504" s="1" t="s">
         <v>56</v>
@@ -6406,26 +6409,26 @@
         <v>141</v>
       </c>
       <c r="B505" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C505">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="506" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A506" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B506" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C506">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="507" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A507" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B507" s="1" t="s">
         <v>30</v>
@@ -6436,13 +6439,13 @@
     </row>
     <row r="508" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A508" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B508" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C508">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="509" spans="1:3" x14ac:dyDescent="0.25">
@@ -6450,10 +6453,10 @@
         <v>142</v>
       </c>
       <c r="B509" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C509">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="510" spans="1:3" x14ac:dyDescent="0.25">
@@ -6461,18 +6464,18 @@
         <v>142</v>
       </c>
       <c r="B510" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C510">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="511" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A511">
-        <v>720004</v>
+      <c r="A511" t="s">
+        <v>142</v>
       </c>
       <c r="B511" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C511">
         <v>70</v>
@@ -6480,21 +6483,21 @@
     </row>
     <row r="512" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A512">
-        <v>720003</v>
+        <v>720004</v>
       </c>
       <c r="B512" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C512">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="513" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A513">
-        <v>720004</v>
+        <v>720003</v>
       </c>
       <c r="B513" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C513">
         <v>0</v>
@@ -6502,7 +6505,7 @@
     </row>
     <row r="514" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A514">
-        <v>720003</v>
+        <v>720004</v>
       </c>
       <c r="B514" s="1" t="s">
         <v>30</v>
@@ -6516,7 +6519,7 @@
         <v>720003</v>
       </c>
       <c r="B515" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C515">
         <v>0</v>
@@ -6524,7 +6527,7 @@
     </row>
     <row r="516" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A516">
-        <v>720004</v>
+        <v>720003</v>
       </c>
       <c r="B516" s="1" t="s">
         <v>1</v>
@@ -6535,13 +6538,13 @@
     </row>
     <row r="517" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A517">
-        <v>721001</v>
+        <v>720004</v>
       </c>
       <c r="B517" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C517">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="518" spans="1:3" x14ac:dyDescent="0.25">
@@ -6549,10 +6552,10 @@
         <v>721001</v>
       </c>
       <c r="B518" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C518">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="519" spans="1:3" x14ac:dyDescent="0.25">
@@ -6560,7 +6563,7 @@
         <v>721001</v>
       </c>
       <c r="B519" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C519">
         <v>0</v>
@@ -6568,13 +6571,13 @@
     </row>
     <row r="520" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A520">
-        <v>651030</v>
+        <v>721001</v>
       </c>
       <c r="B520" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C520">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="521" spans="1:3" x14ac:dyDescent="0.25">
@@ -6582,21 +6585,21 @@
         <v>651030</v>
       </c>
       <c r="B521" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C521">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="522" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A522">
-        <v>651010</v>
+        <v>651030</v>
       </c>
       <c r="B522" s="1" t="s">
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="C522">
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="523" spans="1:3" x14ac:dyDescent="0.25">
@@ -6604,37 +6607,37 @@
         <v>651010</v>
       </c>
       <c r="B523" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C523">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="524" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A524" t="s">
-        <v>143</v>
+      <c r="A524">
+        <v>651010</v>
       </c>
       <c r="B524" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C524">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="525" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A525" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B525" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C525">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="526" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A526" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B526" s="1" t="s">
         <v>1</v>
@@ -6645,7 +6648,7 @@
     </row>
     <row r="527" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A527" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B527" s="1" t="s">
         <v>1</v>
@@ -6656,10 +6659,10 @@
     </row>
     <row r="528" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A528" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B528" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C528">
         <v>0</v>
@@ -6667,7 +6670,7 @@
     </row>
     <row r="529" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A529" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B529" s="1" t="s">
         <v>56</v>
@@ -6678,7 +6681,7 @@
     </row>
     <row r="530" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A530" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B530" s="1" t="s">
         <v>56</v>
@@ -6689,7 +6692,7 @@
     </row>
     <row r="531" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A531" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B531" s="1" t="s">
         <v>56</v>
@@ -6700,10 +6703,10 @@
     </row>
     <row r="532" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A532" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B532" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C532">
         <v>0</v>
@@ -6711,7 +6714,7 @@
     </row>
     <row r="533" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A533" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B533" s="1" t="s">
         <v>30</v>
@@ -6722,7 +6725,7 @@
     </row>
     <row r="534" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A534" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B534" s="1" t="s">
         <v>30</v>
@@ -6733,7 +6736,7 @@
     </row>
     <row r="535" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A535" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B535" s="1" t="s">
         <v>30</v>
@@ -6744,32 +6747,32 @@
     </row>
     <row r="536" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A536" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B536" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C536">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="537" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A537" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B537" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C537">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="538" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A538" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B538" s="1" t="s">
-        <v>56</v>
+        <v>1</v>
       </c>
       <c r="C538">
         <v>0</v>
@@ -6777,7 +6780,7 @@
     </row>
     <row r="539" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A539" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B539" s="1" t="s">
         <v>56</v>
@@ -6788,10 +6791,10 @@
     </row>
     <row r="540" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A540" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B540" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C540">
         <v>0</v>
@@ -6799,7 +6802,7 @@
     </row>
     <row r="541" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A541" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B541" s="1" t="s">
         <v>30</v>
@@ -6810,24 +6813,24 @@
     </row>
     <row r="542" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A542" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B542" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C542">
-        <v>110</v>
+        <v>0</v>
       </c>
     </row>
     <row r="543" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A543" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B543" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C543">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="544" spans="1:3" x14ac:dyDescent="0.25">
@@ -6835,32 +6838,32 @@
         <v>150</v>
       </c>
       <c r="B544" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C544">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="545" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A545" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B545" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C545">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="546" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A546" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B546" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C546">
-        <v>150</v>
+        <v>60</v>
       </c>
     </row>
     <row r="547" spans="1:3" x14ac:dyDescent="0.25">
@@ -6868,18 +6871,18 @@
         <v>151</v>
       </c>
       <c r="B547" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C547">
-        <v>110</v>
+        <v>150</v>
       </c>
     </row>
     <row r="548" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A548">
-        <v>721014</v>
+      <c r="A548" t="s">
+        <v>151</v>
       </c>
       <c r="B548" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C548">
         <v>110</v>
@@ -6887,24 +6890,24 @@
     </row>
     <row r="549" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A549">
-        <v>721008</v>
+        <v>721014</v>
       </c>
       <c r="B549" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C549">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="550" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A550">
-        <v>721005</v>
+        <v>721008</v>
       </c>
       <c r="B550" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C550">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="551" spans="1:3" x14ac:dyDescent="0.25">
@@ -6912,15 +6915,15 @@
         <v>721005</v>
       </c>
       <c r="B551" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C551">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="552" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A552">
-        <v>721008</v>
+        <v>721005</v>
       </c>
       <c r="B552" s="1" t="s">
         <v>1</v>
@@ -6931,24 +6934,24 @@
     </row>
     <row r="553" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A553">
+        <v>721008</v>
+      </c>
+      <c r="B553" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C553">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="554" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A554">
         <v>721014</v>
       </c>
-      <c r="B553" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C553">
+      <c r="B554" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C554">
         <v>50</v>
-      </c>
-    </row>
-    <row r="554" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A554" t="s">
-        <v>152</v>
-      </c>
-      <c r="B554" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C554">
-        <v>110</v>
       </c>
     </row>
     <row r="555" spans="1:3" x14ac:dyDescent="0.25">
@@ -6956,32 +6959,32 @@
         <v>152</v>
       </c>
       <c r="B555" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C555">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="556" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A556" t="s">
+        <v>152</v>
+      </c>
+      <c r="B556" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C556">
         <v>60</v>
       </c>
     </row>
-    <row r="556" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A556">
+    <row r="557" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A557">
         <v>241040</v>
       </c>
-      <c r="B556" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C556">
+      <c r="B557" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C557">
         <v>120</v>
-      </c>
-    </row>
-    <row r="557" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A557">
-        <v>241020</v>
-      </c>
-      <c r="B557" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C557">
-        <v>70</v>
       </c>
     </row>
     <row r="558" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -6989,43 +6992,43 @@
         <v>241020</v>
       </c>
       <c r="B558" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C558">
-        <v>110</v>
+        <v>70</v>
       </c>
     </row>
     <row r="559" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A559">
-        <v>241040</v>
+        <v>241020</v>
       </c>
       <c r="B559" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C559">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="560" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A560">
-        <v>601138</v>
+        <v>241040</v>
       </c>
       <c r="B560" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C560">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="561" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A561">
-        <v>601128</v>
+        <v>601138</v>
       </c>
       <c r="B561" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C561">
-        <v>80</v>
+        <v>110</v>
       </c>
     </row>
     <row r="562" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7033,54 +7036,54 @@
         <v>601128</v>
       </c>
       <c r="B562" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C562">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A563">
+        <v>601128</v>
+      </c>
+      <c r="B563" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C563">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A564">
         <v>601138</v>
       </c>
-      <c r="B563" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C563">
+      <c r="B564" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C564">
         <v>60</v>
-      </c>
-    </row>
-    <row r="564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A564" t="s">
-        <v>153</v>
-      </c>
-      <c r="B564" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C564">
-        <v>120</v>
       </c>
     </row>
     <row r="565" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A565" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B565" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C565">
-        <v>70</v>
+        <v>120</v>
       </c>
     </row>
     <row r="566" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A566" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B566" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C566">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="567" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7088,31 +7091,42 @@
         <v>155</v>
       </c>
       <c r="B567" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C567">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="568" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A568" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B568" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C568">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="569" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A569" t="s">
+        <v>154</v>
+      </c>
+      <c r="B569" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C569">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="570" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A570" t="s">
         <v>153</v>
       </c>
-      <c r="B569" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C569">
+      <c r="B570" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C570">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adding missing material on side 0020 to the config file
</commit_message>
<xml_diff>
--- a/project/config/profile_config_file.xlsx
+++ b/project/config/profile_config_file.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsochacki\Desktop\Python\Tkinter\production-counting\project\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E87D85B-1814-4175-B9A0-F3CB796D2D98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5EA2EF0-9E7C-47E4-9F6B-95617B5B5CF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-195" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="29805" yWindow="615" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="profile_config" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" refMode="R1C1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="874" uniqueCount="178">
   <si>
     <t>GP8280</t>
   </si>
@@ -854,7 +854,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C575"/>
+  <dimension ref="A1:C576"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" customWidth="1"/>
@@ -6860,18 +6860,18 @@
     </row>
     <row r="546" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A546" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B546" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C546">
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="547" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A547" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B547" s="1" t="s">
         <v>30</v>
@@ -6882,24 +6882,24 @@
     </row>
     <row r="548" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A548" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B548" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C548">
-        <v>110</v>
+        <v>0</v>
       </c>
     </row>
     <row r="549" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A549" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B549" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C549">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="550" spans="1:3" x14ac:dyDescent="0.25">
@@ -6907,32 +6907,32 @@
         <v>150</v>
       </c>
       <c r="B550" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C550">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="551" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A551" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B551" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C551">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="552" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A552" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B552" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C552">
-        <v>150</v>
+        <v>60</v>
       </c>
     </row>
     <row r="553" spans="1:3" x14ac:dyDescent="0.25">
@@ -6940,18 +6940,18 @@
         <v>151</v>
       </c>
       <c r="B553" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C553">
-        <v>110</v>
+        <v>150</v>
       </c>
     </row>
     <row r="554" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A554">
-        <v>721014</v>
+      <c r="A554" t="s">
+        <v>151</v>
       </c>
       <c r="B554" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C554">
         <v>110</v>
@@ -6959,24 +6959,24 @@
     </row>
     <row r="555" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A555">
-        <v>721008</v>
+        <v>721014</v>
       </c>
       <c r="B555" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C555">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="556" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A556">
-        <v>721005</v>
+        <v>721008</v>
       </c>
       <c r="B556" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C556">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="557" spans="1:3" x14ac:dyDescent="0.25">
@@ -6984,15 +6984,15 @@
         <v>721005</v>
       </c>
       <c r="B557" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C557">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="558" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A558">
-        <v>721008</v>
+        <v>721005</v>
       </c>
       <c r="B558" s="1" t="s">
         <v>1</v>
@@ -7003,24 +7003,24 @@
     </row>
     <row r="559" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A559">
+        <v>721008</v>
+      </c>
+      <c r="B559" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C559">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="560" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A560">
         <v>721014</v>
       </c>
-      <c r="B559" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C559">
+      <c r="B560" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C560">
         <v>50</v>
-      </c>
-    </row>
-    <row r="560" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A560" t="s">
-        <v>152</v>
-      </c>
-      <c r="B560" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C560">
-        <v>110</v>
       </c>
     </row>
     <row r="561" spans="1:3" x14ac:dyDescent="0.25">
@@ -7028,32 +7028,32 @@
         <v>152</v>
       </c>
       <c r="B561" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C561">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="562" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A562" t="s">
+        <v>152</v>
+      </c>
+      <c r="B562" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C562">
         <v>60</v>
       </c>
     </row>
-    <row r="562" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A562">
+    <row r="563" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A563">
         <v>241040</v>
       </c>
-      <c r="B562" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C562">
+      <c r="B563" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C563">
         <v>120</v>
-      </c>
-    </row>
-    <row r="563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A563">
-        <v>241020</v>
-      </c>
-      <c r="B563" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C563">
-        <v>70</v>
       </c>
     </row>
     <row r="564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7061,43 +7061,43 @@
         <v>241020</v>
       </c>
       <c r="B564" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C564">
-        <v>110</v>
+        <v>70</v>
       </c>
     </row>
     <row r="565" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A565">
-        <v>241040</v>
+        <v>241020</v>
       </c>
       <c r="B565" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C565">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="566" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A566">
-        <v>601138</v>
+        <v>241040</v>
       </c>
       <c r="B566" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C566">
-        <v>110</v>
+        <v>60</v>
       </c>
     </row>
     <row r="567" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A567">
-        <v>601128</v>
+        <v>601138</v>
       </c>
       <c r="B567" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C567">
-        <v>80</v>
+        <v>110</v>
       </c>
     </row>
     <row r="568" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7105,54 +7105,54 @@
         <v>601128</v>
       </c>
       <c r="B568" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C568">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="569" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A569">
+        <v>601128</v>
+      </c>
+      <c r="B569" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C569">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="570" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A570">
         <v>601138</v>
       </c>
-      <c r="B569" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C569">
+      <c r="B570" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C570">
         <v>60</v>
-      </c>
-    </row>
-    <row r="570" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A570" t="s">
-        <v>153</v>
-      </c>
-      <c r="B570" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C570">
-        <v>120</v>
       </c>
     </row>
     <row r="571" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A571" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B571" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C571">
-        <v>70</v>
+        <v>120</v>
       </c>
     </row>
     <row r="572" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A572" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B572" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C572">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="573" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7160,31 +7160,42 @@
         <v>155</v>
       </c>
       <c r="B573" s="1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="C573">
-        <v>90</v>
+        <v>0</v>
       </c>
     </row>
     <row r="574" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A574" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B574" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C574">
-        <v>0</v>
+        <v>90</v>
       </c>
     </row>
     <row r="575" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A575" t="s">
+        <v>154</v>
+      </c>
+      <c r="B575" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C575">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="576" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A576" t="s">
         <v>153</v>
       </c>
-      <c r="B575" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C575">
+      <c r="B576" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C576">
         <v>50</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: correction side of the material
</commit_message>
<xml_diff>
--- a/project/config/profile_config_file.xlsx
+++ b/project/config/profile_config_file.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsochacki\Desktop\Python\Tkinter\production-counting\project\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5EA2EF0-9E7C-47E4-9F6B-95617B5B5CF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C884B0AA-0F22-46F7-A2B4-E9058805DE53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29805" yWindow="615" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-195" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="profile_config" sheetId="1" r:id="rId1"/>
@@ -2320,7 +2320,7 @@
         <v>761016</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C133">
         <v>120</v>
@@ -2782,7 +2782,7 @@
         <v>406323</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C175">
         <v>90</v>
@@ -2969,7 +2969,7 @@
         <v>406215</v>
       </c>
       <c r="B192" s="1" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
       <c r="C192">
         <v>90</v>

</xml_diff>

<commit_message>
fix: side of the material has been correct
</commit_message>
<xml_diff>
--- a/project/config/profile_config_file.xlsx
+++ b/project/config/profile_config_file.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsochacki\Desktop\Python\Tkinter\production-counting\project\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C884B0AA-0F22-46F7-A2B4-E9058805DE53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D815B97-F4EC-4074-8755-E62DC1FE79DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-195" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5081,7 +5081,7 @@
         <v>406010</v>
       </c>
       <c r="B384" s="1" t="s">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="C384">
         <v>120</v>

</xml_diff>